<commit_message>
exports: colonne URSSAF ajoutee aux deux classeurs
Liste de vente : PRIX, URSSAF 12,4 %, Reste apres URSSAF — le montant a
provisionner des l'encaissement apparait sur chaque ligne.

Classeur de stock, feuille Prix : colonne URSSAF intercalee entre le
prix de vente et la marge.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -17,9 +17,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0 &quot;€&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00 &quot;€&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +57,17 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00C0392B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -124,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -137,10 +148,22 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -156,6 +179,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -524,14 +550,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -544,7 +572,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Une ligne = une annonce. Coche la colonne « Fait » au fur et à mesure.</t>
+          <t>Une ligne = une annonce. La colonne URSSAF est le montant à provisionner dès l'encaissement.</t>
         </is>
       </c>
     </row>
@@ -561,15 +589,25 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>URSSAF 12,4 %</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Reste après URSSAF</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>Où le vendre</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -585,6 +623,8 @@
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -595,34 +635,50 @@
       <c r="B6" s="7" t="n">
         <v>139</v>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="8">
+        <f>B6*0.124</f>
+        <v/>
+      </c>
+      <c r="D6" s="9">
+        <f>B6-C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>Texte d'annonce prêt · plancher 129 €</t>
         </is>
       </c>
-      <c r="E6" s="9" t="n"/>
+      <c r="G6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Short ba&amp;sh Fegor lightusedblue — T.34</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="13" t="n">
         <v>75</v>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="14">
+        <f>B7*0.124</f>
+        <v/>
+      </c>
+      <c r="D7" s="15">
+        <f>B7-C7</f>
+        <v/>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr"/>
-      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="16" t="inlineStr"/>
+      <c r="G7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -633,38 +689,54 @@
       <c r="B8" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="8">
+        <f>B8*0.124</f>
+        <v/>
+      </c>
+      <c r="D8" s="9">
+        <f>B8-C8</f>
+        <v/>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + Vinted</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>Vérifier marquage CE et notice FR</t>
         </is>
       </c>
-      <c r="E8" s="9" t="n"/>
+      <c r="G8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle vichy</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="13" t="n">
         <v>19</v>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="14">
+        <f>B9*0.124</f>
+        <v/>
+      </c>
+      <c r="D9" s="15">
+        <f>B9-C9</f>
+        <v/>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + Vinted</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>Vérifier marquage CE et notice FR</t>
         </is>
       </c>
-      <c r="E9" s="13" t="n"/>
+      <c r="G9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -675,49 +747,67 @@
       <c r="B10" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="8">
+        <f>B10*0.124</f>
+        <v/>
+      </c>
+      <c r="D10" s="9">
+        <f>B10-C10</f>
+        <v/>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + Vinted</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>À publier quand le 1ᵉʳ est vendu</t>
         </is>
       </c>
-      <c r="E10" s="9" t="n"/>
+      <c r="G10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ vichy</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="13" t="n">
         <v>19</v>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="14">
+        <f>B11*0.124</f>
+        <v/>
+      </c>
+      <c r="D11" s="15">
+        <f>B11-C11</f>
+        <v/>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + Vinted</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>À publier quand le 1ᵉʳ est vendu</t>
         </is>
       </c>
-      <c r="E11" s="13" t="n"/>
+      <c r="G11" s="17" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>2. À PUBLIER MAINTENANT — les pièces qui rapportent</t>
         </is>
       </c>
-      <c r="B12" s="15" t="n"/>
-      <c r="C12" s="15" t="n"/>
-      <c r="D12" s="15" t="n"/>
-      <c r="E12" s="15" t="n"/>
+      <c r="B12" s="19" t="n"/>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="19" t="n"/>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="19" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -728,38 +818,54 @@
       <c r="B13" s="7" t="n">
         <v>159</v>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="8">
+        <f>B13*0.124</f>
+        <v/>
+      </c>
+      <c r="D13" s="9">
+        <f>B13-C13</f>
+        <v/>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Boutique + Vinted + Leboncoin</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>À recevoir</t>
         </is>
       </c>
-      <c r="E13" s="9" t="n"/>
+      <c r="G13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>BMW Overall ProRain unisexe noir — XL</t>
         </is>
       </c>
-      <c r="B14" s="11" t="n">
+      <c r="B14" s="13" t="n">
         <v>139</v>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="14">
+        <f>B14*0.124</f>
+        <v/>
+      </c>
+      <c r="D14" s="15">
+        <f>B14-C14</f>
+        <v/>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + Vinted</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>À recevoir</t>
         </is>
       </c>
-      <c r="E14" s="13" t="n"/>
+      <c r="G14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -770,38 +876,54 @@
       <c r="B15" s="7" t="n">
         <v>109</v>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="8">
+        <f>B15*0.124</f>
+        <v/>
+      </c>
+      <c r="D15" s="9">
+        <f>B15-C15</f>
+        <v/>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t>Saison rando : sept-nov</t>
         </is>
       </c>
-      <c r="E15" s="9" t="n"/>
+      <c r="G15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Robe Elisabetta Franchi ivoire — 46 IT / 42 FR</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="13" t="n">
         <v>99</v>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="14">
+        <f>B16*0.124</f>
+        <v/>
+      </c>
+      <c r="D16" s="15">
+        <f>B16-C16</f>
+        <v/>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>Défroisser avant photos</t>
         </is>
       </c>
-      <c r="E16" s="13" t="n"/>
+      <c r="G16" s="17" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -812,38 +934,54 @@
       <c r="B17" s="7" t="n">
         <v>99</v>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="8">
+        <f>B17*0.124</f>
+        <v/>
+      </c>
+      <c r="D17" s="9">
+        <f>B17-C17</f>
+        <v/>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="F17" s="10" t="inlineStr">
         <is>
           <t>Vérifier composition sur l'étiquette</t>
         </is>
       </c>
-      <c r="E17" s="9" t="n"/>
+      <c r="G17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Blazer Karl Lagerfeld punto noir — 36 FR / IT 40</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="13" t="n">
         <v>89</v>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C18" s="14">
+        <f>B18*0.124</f>
+        <v/>
+      </c>
+      <c r="D18" s="15">
+        <f>B18-C18</f>
+        <v/>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="F18" s="16" t="inlineStr">
         <is>
           <t>Indiquer les deux tailles</t>
         </is>
       </c>
-      <c r="E18" s="13" t="n"/>
+      <c r="G18" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -854,38 +992,54 @@
       <c r="B19" s="7" t="n">
         <v>89</v>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="8">
+        <f>B19*0.124</f>
+        <v/>
+      </c>
+      <c r="D19" s="9">
+        <f>B19-C19</f>
+        <v/>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>eBay + Leboncoin</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>Une annonce par paire</t>
         </is>
       </c>
-      <c r="E19" s="9" t="n"/>
+      <c r="G19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Adidas Predator Edge.1 TF — 48⅔ — 2ᵉ paire</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="13" t="n">
         <v>89</v>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="14">
+        <f>B20*0.124</f>
+        <v/>
+      </c>
+      <c r="D20" s="15">
+        <f>B20-C20</f>
+        <v/>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>eBay + Leboncoin</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="F20" s="16" t="inlineStr">
         <is>
           <t>Une annonce par paire</t>
         </is>
       </c>
-      <c r="E20" s="13" t="n"/>
+      <c r="G20" s="17" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -896,38 +1050,54 @@
       <c r="B21" s="7" t="n">
         <v>89</v>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="8">
+        <f>B21*0.124</f>
+        <v/>
+      </c>
+      <c r="D21" s="9">
+        <f>B21-C21</f>
+        <v/>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="F21" s="10" t="inlineStr">
         <is>
           <t>Retirer de Vinted d'abord</t>
         </is>
       </c>
-      <c r="E21" s="9" t="n"/>
+      <c r="G21" s="11" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>Plein Sport montante blanc / violet — 40</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="13" t="n">
         <v>89</v>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C22" s="14">
+        <f>B22*0.124</f>
+        <v/>
+      </c>
+      <c r="D22" s="15">
+        <f>B22-C22</f>
+        <v/>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>99 € pendant 2 semaines, puis 89 €</t>
         </is>
       </c>
-      <c r="E22" s="13" t="n"/>
+      <c r="G22" s="17" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -938,30 +1108,46 @@
       <c r="B23" s="7" t="n">
         <v>79</v>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="8">
+        <f>B23*0.124</f>
+        <v/>
+      </c>
+      <c r="D23" s="9">
+        <f>B23-C23</f>
+        <v/>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr"/>
-      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="10" t="inlineStr"/>
+      <c r="G23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Baskets adidas by Stella McCartney UB21 — 36</t>
         </is>
       </c>
-      <c r="B24" s="11" t="n">
+      <c r="B24" s="13" t="n">
         <v>79</v>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C24" s="14">
+        <f>B24*0.124</f>
+        <v/>
+      </c>
+      <c r="D24" s="15">
+        <f>B24-C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr"/>
-      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="16" t="inlineStr"/>
+      <c r="G24" s="17" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -972,34 +1158,50 @@
       <c r="B25" s="7" t="n">
         <v>69</v>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="8">
+        <f>B25*0.124</f>
+        <v/>
+      </c>
+      <c r="D25" s="9">
+        <f>B25-C25</f>
+        <v/>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr"/>
-      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="10" t="inlineStr"/>
+      <c r="G25" s="11" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Ballerines Massimo Dutti cuir rouge — 40 IT</t>
         </is>
       </c>
-      <c r="B26" s="11" t="n">
+      <c r="B26" s="13" t="n">
         <v>59</v>
       </c>
-      <c r="C26" s="10" t="inlineStr">
+      <c r="C26" s="14">
+        <f>B26*0.124</f>
+        <v/>
+      </c>
+      <c r="D26" s="15">
+        <f>B26-C26</f>
+        <v/>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>Pas Vinted : article neuf</t>
         </is>
       </c>
-      <c r="E26" s="13" t="n"/>
+      <c r="G26" s="17" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -1010,34 +1212,50 @@
       <c r="B27" s="7" t="n">
         <v>59</v>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" s="8">
+        <f>B27*0.124</f>
+        <v/>
+      </c>
+      <c r="D27" s="9">
+        <f>B27-C27</f>
+        <v/>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
+      <c r="F27" s="10" t="inlineStr">
         <is>
           <t>Orthographe : Pier ANTONIO</t>
         </is>
       </c>
-      <c r="E27" s="9" t="n"/>
+      <c r="G27" s="11" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>Baskets Geox gris / argent — 35</t>
         </is>
       </c>
-      <c r="B28" s="11" t="n">
+      <c r="B28" s="13" t="n">
         <v>49</v>
       </c>
-      <c r="C28" s="10" t="inlineStr">
+      <c r="C28" s="14">
+        <f>B28*0.124</f>
+        <v/>
+      </c>
+      <c r="D28" s="15">
+        <f>B28-C28</f>
+        <v/>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr"/>
-      <c r="E28" s="13" t="n"/>
+      <c r="F28" s="16" t="inlineStr"/>
+      <c r="G28" s="17" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -1048,30 +1266,46 @@
       <c r="B29" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C29" s="8">
+        <f>B29*0.124</f>
+        <v/>
+      </c>
+      <c r="D29" s="9">
+        <f>B29-C29</f>
+        <v/>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="D29" s="8" t="inlineStr"/>
-      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="10" t="inlineStr"/>
+      <c r="G29" s="11" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>Morgan — jupe marron</t>
         </is>
       </c>
-      <c r="B30" s="11" t="n">
+      <c r="B30" s="13" t="n">
         <v>19</v>
       </c>
-      <c r="C30" s="10" t="inlineStr">
+      <c r="C30" s="14">
+        <f>B30*0.124</f>
+        <v/>
+      </c>
+      <c r="D30" s="15">
+        <f>B30-C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr"/>
-      <c r="E30" s="13" t="n"/>
+      <c r="F30" s="16" t="inlineStr"/>
+      <c r="G30" s="17" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -1082,30 +1316,46 @@
       <c r="B31" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="8">
+        <f>B31*0.124</f>
+        <v/>
+      </c>
+      <c r="D31" s="9">
+        <f>B31-C31</f>
+        <v/>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="D31" s="8" t="inlineStr"/>
-      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="10" t="inlineStr"/>
+      <c r="G31" s="11" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>Morgan — polo rouge à écusson doré L</t>
         </is>
       </c>
-      <c r="B32" s="11" t="n">
+      <c r="B32" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="C32" s="10" t="inlineStr">
+      <c r="C32" s="14">
+        <f>B32*0.124</f>
+        <v/>
+      </c>
+      <c r="D32" s="15">
+        <f>B32-C32</f>
+        <v/>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr"/>
-      <c r="E32" s="13" t="n"/>
+      <c r="F32" s="16" t="inlineStr"/>
+      <c r="G32" s="17" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -1116,41 +1366,59 @@
       <c r="B33" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C33" s="8">
+        <f>B33*0.124</f>
+        <v/>
+      </c>
+      <c r="D33" s="9">
+        <f>B33-C33</f>
+        <v/>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="D33" s="8" t="inlineStr"/>
-      <c r="E33" s="9" t="n"/>
+      <c r="F33" s="10" t="inlineStr"/>
+      <c r="G33" s="11" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>Morgan — polo blanc L</t>
         </is>
       </c>
-      <c r="B34" s="11" t="n">
+      <c r="B34" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="C34" s="10" t="inlineStr">
+      <c r="C34" s="14">
+        <f>B34*0.124</f>
+        <v/>
+      </c>
+      <c r="D34" s="15">
+        <f>B34-C34</f>
+        <v/>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr"/>
-      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="16" t="inlineStr"/>
+      <c r="G34" s="17" t="n"/>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="20" t="inlineStr">
         <is>
           <t>3. LIQUIDER — vendre pour récupérer la trésorerie, pas pour la marge</t>
         </is>
       </c>
-      <c r="B35" s="17" t="n"/>
-      <c r="C35" s="17" t="n"/>
-      <c r="D35" s="17" t="n"/>
-      <c r="E35" s="17" t="n"/>
+      <c r="B35" s="21" t="n"/>
+      <c r="C35" s="21" t="n"/>
+      <c r="D35" s="21" t="n"/>
+      <c r="E35" s="21" t="n"/>
+      <c r="F35" s="21" t="n"/>
+      <c r="G35" s="21" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -1161,34 +1429,50 @@
       <c r="B36" s="7" t="n">
         <v>99</v>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C36" s="8">
+        <f>B36*0.124</f>
+        <v/>
+      </c>
+      <c r="D36" s="9">
+        <f>B36-C36</f>
+        <v/>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="F36" s="10" t="inlineStr">
         <is>
           <t>Préciser « modèle GS », réf. G19064IK</t>
         </is>
       </c>
-      <c r="E36" s="9" t="n"/>
+      <c r="G36" s="11" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="inlineStr">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>Baskets Emporio Armani bleu lavande — 36</t>
         </is>
       </c>
-      <c r="B37" s="11" t="n">
+      <c r="B37" s="13" t="n">
         <v>69</v>
       </c>
-      <c r="C37" s="10" t="inlineStr">
+      <c r="C37" s="14">
+        <f>B37*0.124</f>
+        <v/>
+      </c>
+      <c r="D37" s="15">
+        <f>B37-C37</f>
+        <v/>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="D37" s="12" t="inlineStr"/>
-      <c r="E37" s="13" t="n"/>
+      <c r="F37" s="16" t="inlineStr"/>
+      <c r="G37" s="17" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -1199,30 +1483,46 @@
       <c r="B38" s="7" t="n">
         <v>65</v>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" s="8">
+        <f>B38*0.124</f>
+        <v/>
+      </c>
+      <c r="D38" s="9">
+        <f>B38-C38</f>
+        <v/>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="D38" s="8" t="inlineStr"/>
-      <c r="E38" s="9" t="n"/>
+      <c r="F38" s="10" t="inlineStr"/>
+      <c r="G38" s="11" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>New Balance 650 blanche montante — 44</t>
         </is>
       </c>
-      <c r="B39" s="11" t="n">
+      <c r="B39" s="13" t="n">
         <v>65</v>
       </c>
-      <c r="C39" s="10" t="inlineStr">
+      <c r="C39" s="14">
+        <f>B39*0.124</f>
+        <v/>
+      </c>
+      <c r="D39" s="15">
+        <f>B39-C39</f>
+        <v/>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="D39" s="12" t="inlineStr"/>
-      <c r="E39" s="13" t="n"/>
+      <c r="F39" s="16" t="inlineStr"/>
+      <c r="G39" s="17" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -1233,24 +1533,34 @@
       <c r="B40" s="7" t="n">
         <v>54</v>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C40" s="8">
+        <f>B40*0.124</f>
+        <v/>
+      </c>
+      <c r="D40" s="9">
+        <f>B40-C40</f>
+        <v/>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="D40" s="8" t="inlineStr"/>
-      <c r="E40" s="9" t="n"/>
+      <c r="F40" s="10" t="inlineStr"/>
+      <c r="G40" s="11" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="18" t="inlineStr">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t>4. PLUS TARD — ne pas publier maintenant</t>
         </is>
       </c>
-      <c r="B41" s="19" t="n"/>
-      <c r="C41" s="19" t="n"/>
-      <c r="D41" s="19" t="n"/>
-      <c r="E41" s="19" t="n"/>
+      <c r="B41" s="23" t="n"/>
+      <c r="C41" s="23" t="n"/>
+      <c r="D41" s="23" t="n"/>
+      <c r="E41" s="23" t="n"/>
+      <c r="F41" s="23" t="n"/>
+      <c r="G41" s="23" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -1261,54 +1571,80 @@
       <c r="B42" s="7" t="n">
         <v>199</v>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" s="8">
+        <f>B42*0.124</f>
+        <v/>
+      </c>
+      <c r="D42" s="9">
+        <f>B42-C42</f>
+        <v/>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>Leboncoin B2B</t>
         </is>
       </c>
-      <c r="D42" s="8" t="inlineStr">
+      <c r="F42" s="10" t="inlineStr">
         <is>
           <t>FÉVRIER-MARS, quand le revendeur prépare l'été</t>
         </is>
       </c>
-      <c r="E42" s="9" t="n"/>
+      <c r="G42" s="11" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="10" t="inlineStr">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>Adidas Yeezy 700 V3 Mono Safflower — 38</t>
         </is>
       </c>
-      <c r="B43" s="20" t="inlineStr">
+      <c r="B43" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr">
+      <c r="C43" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D43" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Vinted</t>
         </is>
       </c>
-      <c r="D43" s="12" t="inlineStr">
+      <c r="F43" s="16" t="inlineStr">
         <is>
           <t>BLOQUÉ : authentification requise avant de fixer le prix</t>
         </is>
       </c>
-      <c r="E43" s="13" t="n"/>
+      <c r="G43" s="17" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="21" t="inlineStr">
-        <is>
-          <t>TOTAL — 34 annonces</t>
-        </is>
-      </c>
-      <c r="B44" s="22">
+      <c r="A44" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL — 34 annonces chiffrées</t>
+        </is>
+      </c>
+      <c r="B44" s="26">
         <f>B6+B7+B8+B9+B10+B11+B13+B14+B15+B16+B17+B18+B19+B20+B21+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B36+B37+B38+B39+B40+B42</f>
         <v/>
       </c>
-      <c r="C44" s="23" t="n"/>
-      <c r="D44" s="23" t="n"/>
-      <c r="E44" s="23" t="n"/>
+      <c r="C44" s="27">
+        <f>B44*0.124</f>
+        <v/>
+      </c>
+      <c r="D44" s="26">
+        <f>B44-C44</f>
+        <v/>
+      </c>
+      <c r="E44" s="28" t="n"/>
+      <c r="F44" s="28" t="n"/>
+      <c r="G44" s="28" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1321,6 +1657,13 @@
       <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Règle : ces prix sont déjà calés sous le moins cher trouvé sur Internet. Ne pas les remonter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>URSSAF = 12,3 % de cotisations + 0,1 % de CFP, calculé sur le prix de vente encaissé. À mettre de côté à chaque vente, pas à la fin du trimestre.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
exports: la Salomon marquee vendue dans les deux classeurs
Le markdown avait ete mis a jour, pas les Excel. Corrige :

- Stock complet : prix 100 EUR, frais de carte a 0 (Vinted ne preleve
  rien au vendeur), statut VENDUE, colonne 'Vendu le', fond vert
- Synthese : nouveau bloc 'Ou en est le stock' — CA et marge realises,
  restants, capital encore immobilise
- Feuille Prix : ligne verte
- Liste de vente : section 'VENDU' en tete, la Salomon retiree des
  annonces a publier

Nouveaux totaux : CA 2 368 EUR, marge brute 753,40 EUR, net 601,36 EUR.
Realise : 100 EUR de CA, 22,60 EUR de marge, 65 EUR de capital libere.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -71,7 +71,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -81,6 +81,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001A1A1A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E8449"/>
       </patternFill>
     </fill>
     <fill>
@@ -135,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -156,35 +161,37 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -550,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -616,7 +623,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1. URGENT — à publier cette semaine, la saison finit fin septembre</t>
+          <t>✅ VENDU</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -629,11 +636,11 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Havaianas Slim fuchsia 35/36 — LOT de 10 paires</t>
+          <t>Salomon X Ultra 5 Mid GTX — 44</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="C6" s="8">
         <f>B6*0.124</f>
@@ -645,49 +652,37 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin</t>
+          <t>Vinted, acheteur en Italie</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Texte d'annonce prêt · plancher 129 €</t>
+          <t>Vendue le 12/08 · expédier avant le 19/08 20h12</t>
         </is>
       </c>
       <c r="G6" s="11" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="22" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Short ba&amp;sh Fegor lightusedblue — T.34</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="n">
-        <v>75</v>
-      </c>
-      <c r="C7" s="14">
-        <f>B7*0.124</f>
-        <v/>
-      </c>
-      <c r="D7" s="15">
-        <f>B7-C7</f>
-        <v/>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>Boutique + Leboncoin</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr"/>
-      <c r="G7" s="17" t="n"/>
+          <t>1. URGENT — à publier cette semaine, la saison finit fin septembre</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="13" t="n"/>
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="13" t="n"/>
+      <c r="G7" s="13" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle écru</t>
+          <t>Havaianas Slim fuchsia 35/36 — LOT de 10 paires</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>19</v>
+        <v>139</v>
       </c>
       <c r="C8" s="8">
         <f>B8*0.124</f>
@@ -699,49 +694,45 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin + Vinted</t>
+          <t>Leboncoin</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Vérifier marquage CE et notice FR</t>
+          <t>Texte d'annonce prêt · plancher 129 €</t>
         </is>
       </c>
       <c r="G8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle vichy</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="C9" s="14">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Short ba&amp;sh Fegor lightusedblue — T.34</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>75</v>
+      </c>
+      <c r="C9" s="16">
         <f>B9*0.124</f>
         <v/>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="17">
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Leboncoin + Vinted</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>Vérifier marquage CE et notice FR</t>
-        </is>
-      </c>
-      <c r="G9" s="17" t="n"/>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>Boutique + Leboncoin</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr"/>
+      <c r="G9" s="19" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ écru</t>
+          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle écru</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
@@ -762,119 +753,119 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
+          <t>Vérifier marquage CE et notice FR</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle vichy</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="C11" s="16">
+        <f>B11*0.124</f>
+        <v/>
+      </c>
+      <c r="D11" s="17">
+        <f>B11-C11</f>
+        <v/>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>Leboncoin + Vinted</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>Vérifier marquage CE et notice FR</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ écru</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="C12" s="8">
+        <f>B12*0.124</f>
+        <v/>
+      </c>
+      <c r="D12" s="9">
+        <f>B12-C12</f>
+        <v/>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Leboncoin + Vinted</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
           <t>À publier quand le 1ᵉʳ est vendu</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="G12" s="11" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ vichy</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B13" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="C11" s="14">
-        <f>B11*0.124</f>
-        <v/>
-      </c>
-      <c r="D11" s="15">
-        <f>B11-C11</f>
-        <v/>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="C13" s="16">
+        <f>B13*0.124</f>
+        <v/>
+      </c>
+      <c r="D13" s="17">
+        <f>B13-C13</f>
+        <v/>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Leboncoin + Vinted</t>
         </is>
       </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="F13" s="18" t="inlineStr">
         <is>
           <t>À publier quand le 1ᵉʳ est vendu</t>
         </is>
       </c>
-      <c r="G11" s="17" t="n"/>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="G13" s="19" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>2. À PUBLIER MAINTENANT — les pièces qui rapportent</t>
         </is>
       </c>
-      <c r="B12" s="19" t="n"/>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12" s="19" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Bottes Forma Legacy Waterproof — 45</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>159</v>
-      </c>
-      <c r="C13" s="8">
-        <f>B13*0.124</f>
-        <v/>
-      </c>
-      <c r="D13" s="9">
-        <f>B13-C13</f>
-        <v/>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Boutique + Vinted + Leboncoin</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>À recevoir</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>BMW Overall ProRain unisexe noir — XL</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="n">
-        <v>139</v>
-      </c>
-      <c r="C14" s="14">
-        <f>B14*0.124</f>
-        <v/>
-      </c>
-      <c r="D14" s="15">
-        <f>B14-C14</f>
-        <v/>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>Leboncoin + Vinted</t>
-        </is>
-      </c>
-      <c r="F14" s="16" t="inlineStr">
-        <is>
-          <t>À recevoir</t>
-        </is>
-      </c>
-      <c r="G14" s="17" t="n"/>
+      <c r="B14" s="21" t="n"/>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="21" t="n"/>
+      <c r="G14" s="21" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Salomon X Ultra 5 Mid GTX — 44</t>
+          <t>Bottes Forma Legacy Waterproof — 45</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>109</v>
+        <v>159</v>
       </c>
       <c r="C15" s="8">
         <f>B15*0.124</f>
@@ -886,49 +877,49 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin</t>
+          <t>Boutique + Vinted + Leboncoin</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Saison rando : sept-nov</t>
+          <t>À recevoir</t>
         </is>
       </c>
       <c r="G15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Robe Elisabetta Franchi ivoire — 46 IT / 42 FR</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="n">
-        <v>99</v>
-      </c>
-      <c r="C16" s="14">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>BMW Overall ProRain unisexe noir — XL</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>139</v>
+      </c>
+      <c r="C16" s="16">
         <f>B16*0.124</f>
         <v/>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="17">
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>Boutique</t>
-        </is>
-      </c>
-      <c r="F16" s="16" t="inlineStr">
-        <is>
-          <t>Défroisser avant photos</t>
-        </is>
-      </c>
-      <c r="G16" s="17" t="n"/>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>Leboncoin + Vinted</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>À recevoir</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Jupe Sonia Rykiel midi twill cerises — 34</t>
+          <t>Robe Elisabetta Franchi ivoire — 46 IT / 42 FR</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
@@ -949,44 +940,44 @@
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
+          <t>Défroisser avant photos</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Jupe Sonia Rykiel midi twill cerises — 34</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="n">
+        <v>99</v>
+      </c>
+      <c r="C18" s="16">
+        <f>B18*0.124</f>
+        <v/>
+      </c>
+      <c r="D18" s="17">
+        <f>B18-C18</f>
+        <v/>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>Boutique</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
           <t>Vérifier composition sur l'étiquette</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Blazer Karl Lagerfeld punto noir — 36 FR / IT 40</t>
-        </is>
-      </c>
-      <c r="B18" s="13" t="n">
-        <v>89</v>
-      </c>
-      <c r="C18" s="14">
-        <f>B18*0.124</f>
-        <v/>
-      </c>
-      <c r="D18" s="15">
-        <f>B18-C18</f>
-        <v/>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>Boutique</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>Indiquer les deux tailles</t>
-        </is>
-      </c>
-      <c r="G18" s="17" t="n"/>
+      <c r="G18" s="19" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Adidas Predator Edge.1 TF — 48⅔ — 1ʳᵉ paire</t>
+          <t>Blazer Karl Lagerfeld punto noir — 36 FR / IT 40</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
@@ -1002,49 +993,49 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
+          <t>Boutique</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Indiquer les deux tailles</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Adidas Predator Edge.1 TF — 48⅔ — 1ʳᵉ paire</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="n">
+        <v>89</v>
+      </c>
+      <c r="C20" s="16">
+        <f>B20*0.124</f>
+        <v/>
+      </c>
+      <c r="D20" s="17">
+        <f>B20-C20</f>
+        <v/>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
           <t>eBay + Leboncoin</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F20" s="18" t="inlineStr">
         <is>
           <t>Une annonce par paire</t>
         </is>
       </c>
-      <c r="G19" s="11" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Adidas Predator Edge.1 TF — 48⅔ — 2ᵉ paire</t>
-        </is>
-      </c>
-      <c r="B20" s="13" t="n">
-        <v>89</v>
-      </c>
-      <c r="C20" s="14">
-        <f>B20*0.124</f>
-        <v/>
-      </c>
-      <c r="D20" s="15">
-        <f>B20-C20</f>
-        <v/>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>eBay + Leboncoin</t>
-        </is>
-      </c>
-      <c r="F20" s="16" t="inlineStr">
-        <is>
-          <t>Une annonce par paire</t>
-        </is>
-      </c>
-      <c r="G20" s="17" t="n"/>
+      <c r="G20" s="19" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Robe Sandro Noaim blanche — 40</t>
+          <t>Adidas Predator Edge.1 TF — 48⅔ — 2ᵉ paire</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
@@ -1060,53 +1051,53 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
+          <t>eBay + Leboncoin</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Une annonce par paire</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>Robe Sandro Noaim blanche — 40</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="n">
+        <v>89</v>
+      </c>
+      <c r="C22" s="16">
+        <f>B22*0.124</f>
+        <v/>
+      </c>
+      <c r="D22" s="17">
+        <f>B22-C22</f>
+        <v/>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F22" s="18" t="inlineStr">
         <is>
           <t>Retirer de Vinted d'abord</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>Plein Sport montante blanc / violet — 40</t>
-        </is>
-      </c>
-      <c r="B22" s="13" t="n">
-        <v>89</v>
-      </c>
-      <c r="C22" s="14">
-        <f>B22*0.124</f>
-        <v/>
-      </c>
-      <c r="D22" s="15">
-        <f>B22-C22</f>
-        <v/>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>Leboncoin + eBay</t>
-        </is>
-      </c>
-      <c r="F22" s="16" t="inlineStr">
-        <is>
-          <t>99 € pendant 2 semaines, puis 89 €</t>
-        </is>
-      </c>
-      <c r="G22" s="17" t="n"/>
+      <c r="G22" s="19" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Ballerines Hogan 186 Zeppa Fashion — 36</t>
+          <t>Plein Sport montante blanc / violet — 40</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C23" s="8">
         <f>B23*0.124</f>
@@ -1118,45 +1109,49 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
+          <t>Leboncoin + eBay</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>99 € pendant 2 semaines, puis 89 €</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Ballerines Hogan 186 Zeppa Fashion — 36</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>79</v>
+      </c>
+      <c r="C24" s="16">
+        <f>B24*0.124</f>
+        <v/>
+      </c>
+      <c r="D24" s="17">
+        <f>B24-C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr"/>
-      <c r="G23" s="11" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Baskets adidas by Stella McCartney UB21 — 36</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="n">
-        <v>79</v>
-      </c>
-      <c r="C24" s="14">
-        <f>B24*0.124</f>
-        <v/>
-      </c>
-      <c r="D24" s="15">
-        <f>B24-C24</f>
-        <v/>
-      </c>
-      <c r="E24" s="12" t="inlineStr">
-        <is>
-          <t>Boutique</t>
-        </is>
-      </c>
-      <c r="F24" s="16" t="inlineStr"/>
-      <c r="G24" s="17" t="n"/>
+      <c r="F24" s="18" t="inlineStr"/>
+      <c r="G24" s="19" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Robe bustier Chiara Ferragni noire — M</t>
+          <t>Baskets adidas by Stella McCartney UB21 — 36</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C25" s="8">
         <f>B25*0.124</f>
@@ -1168,45 +1163,41 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Boutique + Leboncoin</t>
+          <t>Boutique</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr"/>
       <c r="G25" s="11" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Ballerines Massimo Dutti cuir rouge — 40 IT</t>
-        </is>
-      </c>
-      <c r="B26" s="13" t="n">
-        <v>59</v>
-      </c>
-      <c r="C26" s="14">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Robe bustier Chiara Ferragni noire — M</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n">
+        <v>69</v>
+      </c>
+      <c r="C26" s="16">
         <f>B26*0.124</f>
         <v/>
       </c>
-      <c r="D26" s="15">
+      <c r="D26" s="17">
         <f>B26-C26</f>
         <v/>
       </c>
-      <c r="E26" s="12" t="inlineStr">
-        <is>
-          <t>Leboncoin + eBay</t>
-        </is>
-      </c>
-      <c r="F26" s="16" t="inlineStr">
-        <is>
-          <t>Pas Vinted : article neuf</t>
-        </is>
-      </c>
-      <c r="G26" s="17" t="n"/>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>Boutique + Leboncoin</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr"/>
+      <c r="G26" s="19" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Robe Pier Antonio Gaspari bleu marine — 42</t>
+          <t>Ballerines Massimo Dutti cuir rouge — 40 IT</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
@@ -1222,49 +1213,53 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
+          <t>Leboncoin + eBay</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Pas Vinted : article neuf</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Robe Pier Antonio Gaspari bleu marine — 42</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="n">
+        <v>59</v>
+      </c>
+      <c r="C28" s="16">
+        <f>B28*0.124</f>
+        <v/>
+      </c>
+      <c r="D28" s="17">
+        <f>B28-C28</f>
+        <v/>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
+      <c r="F28" s="18" t="inlineStr">
         <is>
           <t>Orthographe : Pier ANTONIO</t>
         </is>
       </c>
-      <c r="G27" s="11" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>Baskets Geox gris / argent — 35</t>
-        </is>
-      </c>
-      <c r="B28" s="13" t="n">
-        <v>49</v>
-      </c>
-      <c r="C28" s="14">
-        <f>B28*0.124</f>
-        <v/>
-      </c>
-      <c r="D28" s="15">
-        <f>B28-C28</f>
-        <v/>
-      </c>
-      <c r="E28" s="12" t="inlineStr">
-        <is>
-          <t>Leboncoin + eBay</t>
-        </is>
-      </c>
-      <c r="F28" s="16" t="inlineStr"/>
-      <c r="G28" s="17" t="n"/>
+      <c r="G28" s="19" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Morgan — jean bleu clair T.40</t>
+          <t>Baskets Geox gris / argent — 35</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="C29" s="8">
         <f>B29*0.124</f>
@@ -1283,38 +1278,38 @@
       <c r="G29" s="11" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Morgan — jupe marron</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="n">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Morgan — jean bleu clair T.40</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="C30" s="14">
+      <c r="C30" s="16">
         <f>B30*0.124</f>
         <v/>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="17">
         <f>B30-C30</f>
         <v/>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F30" s="16" t="inlineStr"/>
-      <c r="G30" s="17" t="n"/>
+      <c r="F30" s="18" t="inlineStr"/>
+      <c r="G30" s="19" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Morgan — pantalon blanc T.40</t>
+          <t>Morgan — jupe marron</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C31" s="8">
         <f>B31*0.124</f>
@@ -1333,38 +1328,38 @@
       <c r="G31" s="11" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="inlineStr">
-        <is>
-          <t>Morgan — polo rouge à écusson doré L</t>
-        </is>
-      </c>
-      <c r="B32" s="13" t="n">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>Morgan — pantalon blanc T.40</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="C32" s="14">
+      <c r="C32" s="16">
         <f>B32*0.124</f>
         <v/>
       </c>
-      <c r="D32" s="15">
+      <c r="D32" s="17">
         <f>B32-C32</f>
         <v/>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="14" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F32" s="16" t="inlineStr"/>
-      <c r="G32" s="17" t="n"/>
+      <c r="F32" s="18" t="inlineStr"/>
+      <c r="G32" s="19" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Morgan — top camel lurex L</t>
+          <t>Morgan — polo rouge à écusson doré L</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C33" s="8">
         <f>B33*0.124</f>
@@ -1383,285 +1378,310 @@
       <c r="G33" s="11" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="inlineStr">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>Morgan — top camel lurex L</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="C34" s="16">
+        <f>B34*0.124</f>
+        <v/>
+      </c>
+      <c r="D34" s="17">
+        <f>B34-C34</f>
+        <v/>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>Leboncoin + eBay</t>
+        </is>
+      </c>
+      <c r="F34" s="18" t="inlineStr"/>
+      <c r="G34" s="19" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Morgan — polo blanc L</t>
         </is>
       </c>
-      <c r="B34" s="13" t="n">
+      <c r="B35" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="C34" s="14">
-        <f>B34*0.124</f>
-        <v/>
-      </c>
-      <c r="D34" s="15">
-        <f>B34-C34</f>
-        <v/>
-      </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="C35" s="8">
+        <f>B35*0.124</f>
+        <v/>
+      </c>
+      <c r="D35" s="9">
+        <f>B35-C35</f>
+        <v/>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F34" s="16" t="inlineStr"/>
-      <c r="G34" s="17" t="n"/>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="20" t="inlineStr">
+      <c r="F35" s="10" t="inlineStr"/>
+      <c r="G35" s="11" t="n"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="22" t="inlineStr">
         <is>
           <t>3. LIQUIDER — vendre pour récupérer la trésorerie, pas pour la marge</t>
         </is>
       </c>
-      <c r="B35" s="21" t="n"/>
-      <c r="C35" s="21" t="n"/>
-      <c r="D35" s="21" t="n"/>
-      <c r="E35" s="21" t="n"/>
-      <c r="F35" s="21" t="n"/>
-      <c r="G35" s="21" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="B36" s="23" t="n"/>
+      <c r="C36" s="23" t="n"/>
+      <c r="D36" s="23" t="n"/>
+      <c r="E36" s="23" t="n"/>
+      <c r="F36" s="23" t="n"/>
+      <c r="G36" s="23" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>New Balance GS 1906 Alkaline Green — 38½</t>
         </is>
       </c>
-      <c r="B36" s="7" t="n">
+      <c r="B37" s="7" t="n">
         <v>99</v>
       </c>
-      <c r="C36" s="8">
-        <f>B36*0.124</f>
-        <v/>
-      </c>
-      <c r="D36" s="9">
-        <f>B36-C36</f>
-        <v/>
-      </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="C37" s="8">
+        <f>B37*0.124</f>
+        <v/>
+      </c>
+      <c r="D37" s="9">
+        <f>B37-C37</f>
+        <v/>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="F36" s="10" t="inlineStr">
+      <c r="F37" s="10" t="inlineStr">
         <is>
           <t>Préciser « modèle GS », réf. G19064IK</t>
         </is>
       </c>
-      <c r="G36" s="11" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+      <c r="G37" s="11" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t>Baskets Emporio Armani bleu lavande — 36</t>
         </is>
       </c>
-      <c r="B37" s="13" t="n">
+      <c r="B38" s="15" t="n">
         <v>69</v>
       </c>
-      <c r="C37" s="14">
-        <f>B37*0.124</f>
-        <v/>
-      </c>
-      <c r="D37" s="15">
-        <f>B37-C37</f>
-        <v/>
-      </c>
-      <c r="E37" s="12" t="inlineStr">
+      <c r="C38" s="16">
+        <f>B38*0.124</f>
+        <v/>
+      </c>
+      <c r="D38" s="17">
+        <f>B38-C38</f>
+        <v/>
+      </c>
+      <c r="E38" s="14" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="F37" s="16" t="inlineStr"/>
-      <c r="G37" s="17" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="F38" s="18" t="inlineStr"/>
+      <c r="G38" s="19" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>Tommy Jeans baskets basses noir / blanc — 40</t>
         </is>
       </c>
-      <c r="B38" s="7" t="n">
+      <c r="B39" s="7" t="n">
         <v>65</v>
       </c>
-      <c r="C38" s="8">
-        <f>B38*0.124</f>
-        <v/>
-      </c>
-      <c r="D38" s="9">
-        <f>B38-C38</f>
-        <v/>
-      </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="C39" s="8">
+        <f>B39*0.124</f>
+        <v/>
+      </c>
+      <c r="D39" s="9">
+        <f>B39-C39</f>
+        <v/>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F38" s="10" t="inlineStr"/>
-      <c r="G38" s="11" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="12" t="inlineStr">
+      <c r="F39" s="10" t="inlineStr"/>
+      <c r="G39" s="11" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t>New Balance 650 blanche montante — 44</t>
         </is>
       </c>
-      <c r="B39" s="13" t="n">
+      <c r="B40" s="15" t="n">
         <v>65</v>
       </c>
-      <c r="C39" s="14">
-        <f>B39*0.124</f>
-        <v/>
-      </c>
-      <c r="D39" s="15">
-        <f>B39-C39</f>
-        <v/>
-      </c>
-      <c r="E39" s="12" t="inlineStr">
+      <c r="C40" s="16">
+        <f>B40*0.124</f>
+        <v/>
+      </c>
+      <c r="D40" s="17">
+        <f>B40-C40</f>
+        <v/>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="F39" s="16" t="inlineStr"/>
-      <c r="G39" s="17" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="F40" s="18" t="inlineStr"/>
+      <c r="G40" s="19" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>New Balance BB80 blanc / marine — 38</t>
         </is>
       </c>
-      <c r="B40" s="7" t="n">
+      <c r="B41" s="7" t="n">
         <v>54</v>
       </c>
-      <c r="C40" s="8">
-        <f>B40*0.124</f>
-        <v/>
-      </c>
-      <c r="D40" s="9">
-        <f>B40-C40</f>
-        <v/>
-      </c>
-      <c r="E40" s="6" t="inlineStr">
+      <c r="C41" s="8">
+        <f>B41*0.124</f>
+        <v/>
+      </c>
+      <c r="D41" s="9">
+        <f>B41-C41</f>
+        <v/>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="F40" s="10" t="inlineStr"/>
-      <c r="G40" s="11" t="n"/>
-    </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="22" t="inlineStr">
+      <c r="F41" s="10" t="inlineStr"/>
+      <c r="G41" s="11" t="n"/>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="24" t="inlineStr">
         <is>
           <t>4. PLUS TARD — ne pas publier maintenant</t>
         </is>
       </c>
-      <c r="B41" s="23" t="n"/>
-      <c r="C41" s="23" t="n"/>
-      <c r="D41" s="23" t="n"/>
-      <c r="E41" s="23" t="n"/>
-      <c r="F41" s="23" t="n"/>
-      <c r="G41" s="23" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="B42" s="25" t="n"/>
+      <c r="C42" s="25" t="n"/>
+      <c r="D42" s="25" t="n"/>
+      <c r="E42" s="25" t="n"/>
+      <c r="F42" s="25" t="n"/>
+      <c r="G42" s="25" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>Lot 20 sandales et tongs — EN LOT</t>
         </is>
       </c>
-      <c r="B42" s="7" t="n">
+      <c r="B43" s="7" t="n">
         <v>199</v>
       </c>
-      <c r="C42" s="8">
-        <f>B42*0.124</f>
-        <v/>
-      </c>
-      <c r="D42" s="9">
-        <f>B42-C42</f>
-        <v/>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="C43" s="8">
+        <f>B43*0.124</f>
+        <v/>
+      </c>
+      <c r="D43" s="9">
+        <f>B43-C43</f>
+        <v/>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>Leboncoin B2B</t>
         </is>
       </c>
-      <c r="F42" s="10" t="inlineStr">
+      <c r="F43" s="10" t="inlineStr">
         <is>
           <t>FÉVRIER-MARS, quand le revendeur prépare l'été</t>
         </is>
       </c>
-      <c r="G42" s="11" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="12" t="inlineStr">
+      <c r="G43" s="11" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>Adidas Yeezy 700 V3 Mono Safflower — 38</t>
         </is>
       </c>
-      <c r="B43" s="24" t="inlineStr">
+      <c r="B44" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C43" s="24" t="inlineStr">
+      <c r="C44" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D43" s="24" t="inlineStr">
+      <c r="D44" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E43" s="12" t="inlineStr">
+      <c r="E44" s="14" t="inlineStr">
         <is>
           <t>Vinted</t>
         </is>
       </c>
-      <c r="F43" s="16" t="inlineStr">
+      <c r="F44" s="18" t="inlineStr">
         <is>
           <t>BLOQUÉ : authentification requise avant de fixer le prix</t>
         </is>
       </c>
-      <c r="G43" s="17" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="25" t="inlineStr">
+      <c r="G44" s="19" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="27" t="inlineStr">
         <is>
           <t>TOTAL — 34 annonces chiffrées</t>
         </is>
       </c>
-      <c r="B44" s="26">
-        <f>B6+B7+B8+B9+B10+B11+B13+B14+B15+B16+B17+B18+B19+B20+B21+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B36+B37+B38+B39+B40+B42</f>
-        <v/>
-      </c>
-      <c r="C44" s="27">
-        <f>B44*0.124</f>
-        <v/>
-      </c>
-      <c r="D44" s="26">
-        <f>B44-C44</f>
-        <v/>
-      </c>
-      <c r="E44" s="28" t="n"/>
-      <c r="F44" s="28" t="n"/>
-      <c r="G44" s="28" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Le prix de la Yeezy sera fixé après authentification (10-20 €).</t>
-        </is>
-      </c>
+      <c r="B45" s="28">
+        <f>B6+B8+B9+B10+B11+B12+B13+B15+B16+B17+B18+B19+B20+B21+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B35+B37+B38+B39+B40+B41+B43</f>
+        <v/>
+      </c>
+      <c r="C45" s="29">
+        <f>B45*0.124</f>
+        <v/>
+      </c>
+      <c r="D45" s="28">
+        <f>B45-C45</f>
+        <v/>
+      </c>
+      <c r="E45" s="30" t="n"/>
+      <c r="F45" s="30" t="n"/>
+      <c r="G45" s="30" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Règle : ces prix sont déjà calés sous le moins cher trouvé sur Internet. Ne pas les remonter.</t>
+          <t>Le prix de la Yeezy sera fixé après authentification (10-20 €).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Règle : ces prix sont déjà calés sous le moins cher trouvé sur Internet. Ne pas les remonter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>URSSAF = 12,3 % de cotisations + 0,1 % de CFP, calculé sur le prix de vente encaissé. À mettre de côté à chaque vente, pas à la fin du trimestre.</t>
         </is>

</xml_diff>

<commit_message>
stock: ajout des deux pompes Robby VP550W
Lot de 2 adjuge 45 EUR tout compris, soit 22,50 EUR la pompe pour un
article a 54,90 EUR neuf. Prix 39 EUR piece, marge 23,33 EUR, 52 % de
rendement pour deux annonces.

Remise en main propre obligatoire : a 4,8 kg, le port de 12 EUR ferait
passer le total acheteur a 51 EUR contre 54,90 EUR pour du neuf garanti.

Nouveau piege dans la checklist : un article lourd et bon marche ne
s'expedie pas. Quand le port depasse un quart du prix de vente, prevoir
la main propre ou passer son tour.

Capital 1 407,19 EUR, CA 2 446 EUR, marge brute 776,73 EUR.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1280,11 +1280,11 @@
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>Morgan — jean bleu clair T.40</t>
+          <t>Robby VP550W pompe immergée 550 W — 1ʳᵉ</t>
         </is>
       </c>
       <c r="B30" s="15" t="n">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="C30" s="16">
         <f>B30*0.124</f>
@@ -1296,20 +1296,24 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>Leboncoin + eBay</t>
-        </is>
-      </c>
-      <c r="F30" s="18" t="inlineStr"/>
+          <t>Leboncoin, main propre</t>
+        </is>
+      </c>
+      <c r="F30" s="18" t="inlineStr">
+        <is>
+          <t>TESTER avant de publier · pas d'expédition</t>
+        </is>
+      </c>
       <c r="G30" s="19" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Morgan — jupe marron</t>
+          <t>Robby VP550W pompe immergée 550 W — 2ᵉ</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="C31" s="8">
         <f>B31*0.124</f>
@@ -1321,20 +1325,24 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin + eBay</t>
-        </is>
-      </c>
-      <c r="F31" s="10" t="inlineStr"/>
+          <t>Leboncoin, main propre</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>À publier quand la 1ʳᵉ est vendue</t>
+        </is>
+      </c>
       <c r="G31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>Morgan — pantalon blanc T.40</t>
+          <t>Morgan — jean bleu clair T.40</t>
         </is>
       </c>
       <c r="B32" s="15" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C32" s="16">
         <f>B32*0.124</f>
@@ -1355,11 +1363,11 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Morgan — polo rouge à écusson doré L</t>
+          <t>Morgan — jupe marron</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C33" s="8">
         <f>B33*0.124</f>
@@ -1380,11 +1388,11 @@
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>Morgan — top camel lurex L</t>
+          <t>Morgan — pantalon blanc T.40</t>
         </is>
       </c>
       <c r="B34" s="15" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C34" s="16">
         <f>B34*0.124</f>
@@ -1405,11 +1413,11 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Morgan — polo blanc L</t>
+          <t>Morgan — polo rouge à écusson doré L</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C35" s="8">
         <f>B35*0.124</f>
@@ -1427,27 +1435,39 @@
       <c r="F35" s="10" t="inlineStr"/>
       <c r="G35" s="11" t="n"/>
     </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="22" t="inlineStr">
-        <is>
-          <t>3. LIQUIDER — vendre pour récupérer la trésorerie, pas pour la marge</t>
-        </is>
-      </c>
-      <c r="B36" s="23" t="n"/>
-      <c r="C36" s="23" t="n"/>
-      <c r="D36" s="23" t="n"/>
-      <c r="E36" s="23" t="n"/>
-      <c r="F36" s="23" t="n"/>
-      <c r="G36" s="23" t="n"/>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>Morgan — top camel lurex L</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="C36" s="16">
+        <f>B36*0.124</f>
+        <v/>
+      </c>
+      <c r="D36" s="17">
+        <f>B36-C36</f>
+        <v/>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>Leboncoin + eBay</t>
+        </is>
+      </c>
+      <c r="F36" s="18" t="inlineStr"/>
+      <c r="G36" s="19" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>New Balance GS 1906 Alkaline Green — 38½</t>
+          <t>Morgan — polo blanc L</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C37" s="8">
         <f>B37*0.124</f>
@@ -1459,49 +1479,33 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin</t>
-        </is>
-      </c>
-      <c r="F37" s="10" t="inlineStr">
-        <is>
-          <t>Préciser « modèle GS », réf. G19064IK</t>
-        </is>
-      </c>
+          <t>Leboncoin + eBay</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr"/>
       <c r="G37" s="11" t="n"/>
     </row>
-    <row r="38">
-      <c r="A38" s="14" t="inlineStr">
-        <is>
-          <t>Baskets Emporio Armani bleu lavande — 36</t>
-        </is>
-      </c>
-      <c r="B38" s="15" t="n">
-        <v>69</v>
-      </c>
-      <c r="C38" s="16">
-        <f>B38*0.124</f>
-        <v/>
-      </c>
-      <c r="D38" s="17">
-        <f>B38-C38</f>
-        <v/>
-      </c>
-      <c r="E38" s="14" t="inlineStr">
-        <is>
-          <t>Leboncoin</t>
-        </is>
-      </c>
-      <c r="F38" s="18" t="inlineStr"/>
-      <c r="G38" s="19" t="n"/>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>3. LIQUIDER — vendre pour récupérer la trésorerie, pas pour la marge</t>
+        </is>
+      </c>
+      <c r="B38" s="23" t="n"/>
+      <c r="C38" s="23" t="n"/>
+      <c r="D38" s="23" t="n"/>
+      <c r="E38" s="23" t="n"/>
+      <c r="F38" s="23" t="n"/>
+      <c r="G38" s="23" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Tommy Jeans baskets basses noir / blanc — 40</t>
+          <t>New Balance GS 1906 Alkaline Green — 38½</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>65</v>
+        <v>99</v>
       </c>
       <c r="C39" s="8">
         <f>B39*0.124</f>
@@ -1513,20 +1517,24 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin + eBay</t>
-        </is>
-      </c>
-      <c r="F39" s="10" t="inlineStr"/>
+          <t>Leboncoin</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>Préciser « modèle GS », réf. G19064IK</t>
+        </is>
+      </c>
       <c r="G39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>New Balance 650 blanche montante — 44</t>
+          <t>Baskets Emporio Armani bleu lavande — 36</t>
         </is>
       </c>
       <c r="B40" s="15" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C40" s="16">
         <f>B40*0.124</f>
@@ -1547,11 +1555,11 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>New Balance BB80 blanc / marine — 38</t>
+          <t>Tommy Jeans baskets basses noir / blanc — 40</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="C41" s="8">
         <f>B41*0.124</f>
@@ -1563,33 +1571,45 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin</t>
+          <t>Leboncoin + eBay</t>
         </is>
       </c>
       <c r="F41" s="10" t="inlineStr"/>
       <c r="G41" s="11" t="n"/>
     </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="24" t="inlineStr">
-        <is>
-          <t>4. PLUS TARD — ne pas publier maintenant</t>
-        </is>
-      </c>
-      <c r="B42" s="25" t="n"/>
-      <c r="C42" s="25" t="n"/>
-      <c r="D42" s="25" t="n"/>
-      <c r="E42" s="25" t="n"/>
-      <c r="F42" s="25" t="n"/>
-      <c r="G42" s="25" t="n"/>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>New Balance 650 blanche montante — 44</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="n">
+        <v>65</v>
+      </c>
+      <c r="C42" s="16">
+        <f>B42*0.124</f>
+        <v/>
+      </c>
+      <c r="D42" s="17">
+        <f>B42-C42</f>
+        <v/>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>Leboncoin</t>
+        </is>
+      </c>
+      <c r="F42" s="18" t="inlineStr"/>
+      <c r="G42" s="19" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Lot 20 sandales et tongs — EN LOT</t>
+          <t>New Balance BB80 blanc / marine — 38</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>199</v>
+        <v>54</v>
       </c>
       <c r="C43" s="8">
         <f>B43*0.124</f>
@@ -1601,87 +1621,125 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
+          <t>Leboncoin</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr"/>
+      <c r="G43" s="11" t="n"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="24" t="inlineStr">
+        <is>
+          <t>4. PLUS TARD — ne pas publier maintenant</t>
+        </is>
+      </c>
+      <c r="B44" s="25" t="n"/>
+      <c r="C44" s="25" t="n"/>
+      <c r="D44" s="25" t="n"/>
+      <c r="E44" s="25" t="n"/>
+      <c r="F44" s="25" t="n"/>
+      <c r="G44" s="25" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Lot 20 sandales et tongs — EN LOT</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="n">
+        <v>199</v>
+      </c>
+      <c r="C45" s="8">
+        <f>B45*0.124</f>
+        <v/>
+      </c>
+      <c r="D45" s="9">
+        <f>B45-C45</f>
+        <v/>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
           <t>Leboncoin B2B</t>
         </is>
       </c>
-      <c r="F43" s="10" t="inlineStr">
+      <c r="F45" s="10" t="inlineStr">
         <is>
           <t>FÉVRIER-MARS, quand le revendeur prépare l'été</t>
         </is>
       </c>
-      <c r="G43" s="11" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="14" t="inlineStr">
+      <c r="G45" s="11" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>Adidas Yeezy 700 V3 Mono Safflower — 38</t>
         </is>
       </c>
-      <c r="B44" s="26" t="inlineStr">
+      <c r="B46" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C44" s="26" t="inlineStr">
+      <c r="C46" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D44" s="26" t="inlineStr">
+      <c r="D46" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr">
+      <c r="E46" s="14" t="inlineStr">
         <is>
           <t>Vinted</t>
         </is>
       </c>
-      <c r="F44" s="18" t="inlineStr">
+      <c r="F46" s="18" t="inlineStr">
         <is>
           <t>BLOQUÉ : authentification requise avant de fixer le prix</t>
         </is>
       </c>
-      <c r="G44" s="19" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="27" t="inlineStr">
-        <is>
-          <t>TOTAL — 34 annonces chiffrées</t>
-        </is>
-      </c>
-      <c r="B45" s="28">
-        <f>B6+B8+B9+B10+B11+B12+B13+B15+B16+B17+B18+B19+B20+B21+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B35+B37+B38+B39+B40+B41+B43</f>
-        <v/>
-      </c>
-      <c r="C45" s="29">
-        <f>B45*0.124</f>
-        <v/>
-      </c>
-      <c r="D45" s="28">
-        <f>B45-C45</f>
-        <v/>
-      </c>
-      <c r="E45" s="30" t="n"/>
-      <c r="F45" s="30" t="n"/>
-      <c r="G45" s="30" t="n"/>
+      <c r="G46" s="19" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Le prix de la Yeezy sera fixé après authentification (10-20 €).</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Règle : ces prix sont déjà calés sous le moins cher trouvé sur Internet. Ne pas les remonter.</t>
-        </is>
-      </c>
+      <c r="A47" s="27" t="inlineStr">
+        <is>
+          <t>TOTAL — 36 annonces chiffrées</t>
+        </is>
+      </c>
+      <c r="B47" s="28">
+        <f>B6+B8+B9+B10+B11+B12+B13+B15+B16+B17+B18+B19+B20+B21+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36+B37+B39+B40+B41+B42+B43+B45</f>
+        <v/>
+      </c>
+      <c r="C47" s="29">
+        <f>B47*0.124</f>
+        <v/>
+      </c>
+      <c r="D47" s="28">
+        <f>B47-C47</f>
+        <v/>
+      </c>
+      <c r="E47" s="30" t="n"/>
+      <c r="F47" s="30" t="n"/>
+      <c r="G47" s="30" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Le prix de la Yeezy sera fixé après authentification (10-20 €).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Règle : ces prix sont déjà calés sous le moins cher trouvé sur Internet. Ne pas les remonter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>URSSAF = 12,3 % de cotisations + 0,1 % de CFP, calculé sur le prix de vente encaissé. À mettre de côté à chaque vente, pas à la fin du trimestre.</t>
         </is>

</xml_diff>

<commit_message>
stock: les pompes Robby sont neuves, prix a 44 EUR
Reclassement en neuf : prix 44 EUR piece (49 EUR en test 10 jours),
marge 32,09 EUR au lieu de 23,33. Le lot passe 7e au classement.

Remise en main propre encore plus imperative en neuf : expediee a 44 EUR
+ 12 EUR de port, l'offre depasse les 54,90 EUR du neuf garanti en
magasin.

Vendre du neuf engage davantage : garantie legale de 2 ans portee seul
(provision 4-5 EUR par pompe) et obligations DEEE. La maison de vente
les decrivait 'produit d'occasion' — decrire exactement ce qui est
constate en main et conserver la facture.

CA 2 456 EUR, marge brute 785,49 EUR, net 626,14 EUR.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -1280,11 +1280,11 @@
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>Robby VP550W pompe immergée 550 W — 1ʳᵉ</t>
+          <t>Robby VP550W pompe immergée 550 W NEUVE — 1ʳᵉ</t>
         </is>
       </c>
       <c r="B30" s="15" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C30" s="16">
         <f>B30*0.124</f>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="F30" s="18" t="inlineStr">
         <is>
-          <t>TESTER avant de publier · pas d'expédition</t>
+          <t>49 € pendant 10 jours puis 44 € · JAMAIS d'expédition</t>
         </is>
       </c>
       <c r="G30" s="19" t="n"/>
@@ -1309,11 +1309,11 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Robby VP550W pompe immergée 550 W — 2ᵉ</t>
+          <t>Robby VP550W pompe immergée 550 W NEUVE — 2ᵉ</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C31" s="8">
         <f>B31*0.124</f>

</xml_diff>

<commit_message>
stock: pompes Robby a 42 EUR, tres bon etat, et correction DEEE
Prix fige a 42 EUR piece, marge 28,58 EUR. Etat decrit par les faits
plutot que par une categorie : 'jamais utilisee, emballage ouvert,
testee et fonctionnelle'.

Correction : le DEEE ne s'applique pas. L'eco-participation pese sur le
producteur — fabricant, importateur ou premier metteur sur le marche
francais. Revendre des biens deja commercialises fait de nous un
distributeur, pas un producteur.

Ajout a la checklist : la duree de garantie decoule de l'etat reel, pas
de la case cochee.

CA 2 452 EUR, marge brute 781,98 EUR, net 622,76 EUR.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -1280,11 +1280,11 @@
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>Robby VP550W pompe immergée 550 W NEUVE — 1ʳᵉ</t>
+          <t>Robby VP550W pompe immergée 550 W — 1ʳᵉ</t>
         </is>
       </c>
       <c r="B30" s="15" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C30" s="16">
         <f>B30*0.124</f>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="F30" s="18" t="inlineStr">
         <is>
-          <t>49 € pendant 10 jours puis 44 € · JAMAIS d'expédition</t>
+          <t>« Très bon état, jamais utilisée » · JAMAIS d'expédition</t>
         </is>
       </c>
       <c r="G30" s="19" t="n"/>
@@ -1309,11 +1309,11 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Robby VP550W pompe immergée 550 W NEUVE — 2ᵉ</t>
+          <t>Robby VP550W pompe immergée 550 W — 2ᵉ</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C31" s="8">
         <f>B31*0.124</f>

</xml_diff>

<commit_message>
pokemon: facture Meccha Japan integree, prix recalcules sur le marche
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -90,12 +90,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C0392B"/>
+        <fgColor rgb="00F7F7F7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F7F7F7"/>
+        <fgColor rgb="00C0392B"/>
       </patternFill>
     </fill>
     <fill>
@@ -161,19 +161,19 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,7 +181,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -623,7 +623,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>✅ VENDU</t>
+          <t>✅ VENDU — 593 €, dont 493 € encaissés</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -636,11 +636,11 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Salomon X Ultra 5 Mid GTX — 44</t>
+          <t>T-shirt Balenciaga — T.2</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>100</v>
+        <v>135</v>
       </c>
       <c r="C6" s="8">
         <f>B6*0.124</f>
@@ -652,37 +652,53 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
+          <t>Main propre, espèces</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Encaissé le 09/08 · marge +2,49 € seulement</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Salomon X Ultra 5 Mid GTX — 44</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="C7" s="14">
+        <f>B7*0.124</f>
+        <v/>
+      </c>
+      <c r="D7" s="15">
+        <f>B7-C7</f>
+        <v/>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
           <t>Vinted, acheteur en Italie</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>Vendue le 12/08 · expédier avant le 19/08 20h12</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="n"/>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>1. URGENT — à publier cette semaine, la saison finit fin septembre</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="n"/>
-      <c r="C7" s="13" t="n"/>
-      <c r="D7" s="13" t="n"/>
-      <c r="E7" s="13" t="n"/>
-      <c r="F7" s="13" t="n"/>
-      <c r="G7" s="13" t="n"/>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Vendue le 12/08 · EXPÉDIER AVANT LE 19/08 20h12 · non encaissé</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Havaianas Slim fuchsia 35/36 — LOT de 10 paires</t>
+          <t>Baskets Hoka — 37⅓</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>139</v>
+        <v>80</v>
       </c>
       <c r="C8" s="8">
         <f>B8*0.124</f>
@@ -694,49 +710,53 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin</t>
+          <t>Main propre, espèces</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Texte d'annonce prêt · plancher 129 €</t>
+          <t>Encaissé le 09/08</t>
         </is>
       </c>
       <c r="G8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>Short ba&amp;sh Fegor lightusedblue — T.34</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="n">
-        <v>75</v>
-      </c>
-      <c r="C9" s="16">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Sac demi-lune Karl Lagerfeld Jeans</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="C9" s="14">
         <f>B9*0.124</f>
         <v/>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="15">
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>Boutique + Leboncoin</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr"/>
-      <c r="G9" s="19" t="n"/>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Main propre, espèces</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Encaissé le 09/08</t>
+        </is>
+      </c>
+      <c r="G9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle écru</t>
+          <t>Nike Air Max Moto 2K — 44,5</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="C10" s="8">
         <f>B10*0.124</f>
@@ -748,53 +768,53 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin + Vinted</t>
+          <t>Main propre, espèces</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Vérifier marquage CE et notice FR</t>
+          <t>Encaissé le 09/08</t>
         </is>
       </c>
       <c r="G10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle vichy</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="n">
-        <v>19</v>
-      </c>
-      <c r="C11" s="16">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Lacoste sneakers — 42</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="C11" s="14">
         <f>B11*0.124</f>
         <v/>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="15">
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>Leboncoin + Vinted</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>Vérifier marquage CE et notice FR</t>
-        </is>
-      </c>
-      <c r="G11" s="19" t="n"/>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Main propre, espèces</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Encaissé le 09/08 · marge +1,44 € seulement</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ écru</t>
+          <t>Veste en jean Armani Exchange — T.S</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="C12" s="8">
         <f>B12*0.124</f>
@@ -806,66 +826,66 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin + Vinted</t>
+          <t>Main propre, espèces</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>À publier quand le 1ᵉʳ est vendu</t>
+          <t>Encaissé le 09/08</t>
         </is>
       </c>
       <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ vichy</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="n">
-        <v>19</v>
-      </c>
-      <c r="C13" s="16">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Havaianas Slim — 2 paires à 14 €</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>28</v>
+      </c>
+      <c r="C13" s="14">
         <f>B13*0.124</f>
         <v/>
       </c>
-      <c r="D13" s="17">
+      <c r="D13" s="15">
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Leboncoin + Vinted</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>À publier quand le 1ᵉʳ est vendu</t>
-        </is>
-      </c>
-      <c r="G13" s="19" t="n"/>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Main propre, espèces</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Encaissé le 10/08</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="20" t="inlineStr">
-        <is>
-          <t>2. À PUBLIER MAINTENANT — les pièces qui rapportent</t>
-        </is>
-      </c>
-      <c r="B14" s="21" t="n"/>
-      <c r="C14" s="21" t="n"/>
-      <c r="D14" s="21" t="n"/>
-      <c r="E14" s="21" t="n"/>
-      <c r="F14" s="21" t="n"/>
-      <c r="G14" s="21" t="n"/>
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>1. URGENT — à publier cette semaine, la saison finit fin septembre</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="19" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Bottes Forma Legacy Waterproof — 45</t>
+          <t>Havaianas Slim fuchsia 35/36 — LOT de 10 paires</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>159</v>
+        <v>139</v>
       </c>
       <c r="C15" s="8">
         <f>B15*0.124</f>
@@ -877,53 +897,49 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Boutique + Vinted + Leboncoin</t>
+          <t>Leboncoin</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>À recevoir</t>
+          <t>Texte d'annonce prêt · plancher 129 €</t>
         </is>
       </c>
       <c r="G15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>BMW Overall ProRain unisexe noir — XL</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="n">
-        <v>139</v>
-      </c>
-      <c r="C16" s="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Short ba&amp;sh Fegor lightusedblue — T.34</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="n">
+        <v>75</v>
+      </c>
+      <c r="C16" s="14">
         <f>B16*0.124</f>
         <v/>
       </c>
-      <c r="D16" s="17">
+      <c r="D16" s="15">
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>Leboncoin + Vinted</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>À recevoir</t>
-        </is>
-      </c>
-      <c r="G16" s="19" t="n"/>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Boutique + Leboncoin</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr"/>
+      <c r="G16" s="17" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Robe Elisabetta Franchi ivoire — 46 IT / 42 FR</t>
+          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle écru</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>99</v>
+        <v>19</v>
       </c>
       <c r="C17" s="8">
         <f>B17*0.124</f>
@@ -935,53 +951,53 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Boutique</t>
+          <t>Leboncoin + Vinted</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>Défroisser avant photos</t>
+          <t>Vérifier marquage CE et notice FR</t>
         </is>
       </c>
       <c r="G17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Jupe Sonia Rykiel midi twill cerises — 34</t>
-        </is>
-      </c>
-      <c r="B18" s="15" t="n">
-        <v>99</v>
-      </c>
-      <c r="C18" s="16">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle vichy</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C18" s="14">
         <f>B18*0.124</f>
         <v/>
       </c>
-      <c r="D18" s="17">
+      <c r="D18" s="15">
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>Boutique</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Vérifier composition sur l'étiquette</t>
-        </is>
-      </c>
-      <c r="G18" s="19" t="n"/>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Leboncoin + Vinted</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>Vérifier marquage CE et notice FR</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Blazer Karl Lagerfeld punto noir — 36 FR / IT 40</t>
+          <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ écru</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>89</v>
+        <v>19</v>
       </c>
       <c r="C19" s="8">
         <f>B19*0.124</f>
@@ -993,753 +1009,1243 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
+          <t>Leboncoin + Vinted</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>À publier quand le 1ᵉʳ est vendu</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ vichy</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="14">
+        <f>B20*0.124</f>
+        <v/>
+      </c>
+      <c r="D20" s="15">
+        <f>B20-C20</f>
+        <v/>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Leboncoin + Vinted</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>À publier quand le 1ᵉʳ est vendu</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>2. À PUBLIER MAINTENANT — les pièces qui rapportent</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="n"/>
+      <c r="C21" s="21" t="n"/>
+      <c r="D21" s="21" t="n"/>
+      <c r="E21" s="21" t="n"/>
+      <c r="F21" s="21" t="n"/>
+      <c r="G21" s="21" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Bottes Forma Legacy Waterproof — 45</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>159</v>
+      </c>
+      <c r="C22" s="8">
+        <f>B22*0.124</f>
+        <v/>
+      </c>
+      <c r="D22" s="9">
+        <f>B22-C22</f>
+        <v/>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Boutique + Vinted + Leboncoin</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>À recevoir</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>BMW Overall ProRain unisexe noir — XL</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="n">
+        <v>139</v>
+      </c>
+      <c r="C23" s="14">
+        <f>B23*0.124</f>
+        <v/>
+      </c>
+      <c r="D23" s="15">
+        <f>B23-C23</f>
+        <v/>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>Leboncoin + Vinted</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>À recevoir</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Robe Elisabetta Franchi ivoire — 46 IT / 42 FR</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>99</v>
+      </c>
+      <c r="C24" s="8">
+        <f>B24*0.124</f>
+        <v/>
+      </c>
+      <c r="D24" s="9">
+        <f>B24-C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Défroisser avant photos</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Jupe Sonia Rykiel midi twill cerises — 34</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>99</v>
+      </c>
+      <c r="C25" s="14">
+        <f>B25*0.124</f>
+        <v/>
+      </c>
+      <c r="D25" s="15">
+        <f>B25-C25</f>
+        <v/>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>Boutique</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>Vérifier composition sur l'étiquette</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Blazer Karl Lagerfeld punto noir — 36 FR / IT 40</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>89</v>
+      </c>
+      <c r="C26" s="8">
+        <f>B26*0.124</f>
+        <v/>
+      </c>
+      <c r="D26" s="9">
+        <f>B26-C26</f>
+        <v/>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Boutique</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
         <is>
           <t>Indiquer les deux tailles</t>
         </is>
       </c>
-      <c r="G19" s="11" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="G26" s="11" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Adidas Predator Edge.1 TF — 48⅔ — 1ʳᵉ paire</t>
         </is>
       </c>
-      <c r="B20" s="15" t="n">
+      <c r="B27" s="13" t="n">
         <v>89</v>
       </c>
-      <c r="C20" s="16">
-        <f>B20*0.124</f>
-        <v/>
-      </c>
-      <c r="D20" s="17">
-        <f>B20-C20</f>
-        <v/>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="C27" s="14">
+        <f>B27*0.124</f>
+        <v/>
+      </c>
+      <c r="D27" s="15">
+        <f>B27-C27</f>
+        <v/>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>eBay + Leboncoin</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>Une annonce par paire</t>
         </is>
       </c>
-      <c r="G20" s="19" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="G27" s="17" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Adidas Predator Edge.1 TF — 48⅔ — 2ᵉ paire</t>
         </is>
       </c>
-      <c r="B21" s="7" t="n">
+      <c r="B28" s="7" t="n">
         <v>89</v>
       </c>
-      <c r="C21" s="8">
-        <f>B21*0.124</f>
-        <v/>
-      </c>
-      <c r="D21" s="9">
-        <f>B21-C21</f>
-        <v/>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="C28" s="8">
+        <f>B28*0.124</f>
+        <v/>
+      </c>
+      <c r="D28" s="9">
+        <f>B28-C28</f>
+        <v/>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>eBay + Leboncoin</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F28" s="10" t="inlineStr">
         <is>
           <t>Une annonce par paire</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="G28" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>Robe Sandro Noaim blanche — 40</t>
         </is>
       </c>
-      <c r="B22" s="15" t="n">
+      <c r="B29" s="13" t="n">
         <v>89</v>
       </c>
-      <c r="C22" s="16">
-        <f>B22*0.124</f>
-        <v/>
-      </c>
-      <c r="D22" s="17">
-        <f>B22-C22</f>
-        <v/>
-      </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="C29" s="14">
+        <f>B29*0.124</f>
+        <v/>
+      </c>
+      <c r="D29" s="15">
+        <f>B29-C29</f>
+        <v/>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="F22" s="18" t="inlineStr">
+      <c r="F29" s="16" t="inlineStr">
         <is>
           <t>Retirer de Vinted d'abord</t>
         </is>
       </c>
-      <c r="G22" s="19" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="G29" s="17" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Plein Sport montante blanc / violet — 40</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n">
+      <c r="B30" s="7" t="n">
         <v>89</v>
       </c>
-      <c r="C23" s="8">
-        <f>B23*0.124</f>
-        <v/>
-      </c>
-      <c r="D23" s="9">
-        <f>B23-C23</f>
-        <v/>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="C30" s="8">
+        <f>B30*0.124</f>
+        <v/>
+      </c>
+      <c r="D30" s="9">
+        <f>B30-C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
+      <c r="F30" s="10" t="inlineStr">
         <is>
           <t>99 € pendant 2 semaines, puis 89 €</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="G30" s="11" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>Ballerines Hogan 186 Zeppa Fashion — 36</t>
         </is>
       </c>
-      <c r="B24" s="15" t="n">
+      <c r="B31" s="13" t="n">
         <v>79</v>
       </c>
-      <c r="C24" s="16">
-        <f>B24*0.124</f>
-        <v/>
-      </c>
-      <c r="D24" s="17">
-        <f>B24-C24</f>
-        <v/>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="C31" s="14">
+        <f>B31*0.124</f>
+        <v/>
+      </c>
+      <c r="D31" s="15">
+        <f>B31-C31</f>
+        <v/>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="F24" s="18" t="inlineStr"/>
-      <c r="G24" s="19" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="F31" s="16" t="inlineStr"/>
+      <c r="G31" s="17" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>Baskets adidas by Stella McCartney UB21 — 36</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n">
+      <c r="B32" s="7" t="n">
         <v>79</v>
       </c>
-      <c r="C25" s="8">
-        <f>B25*0.124</f>
-        <v/>
-      </c>
-      <c r="D25" s="9">
-        <f>B25-C25</f>
-        <v/>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="C32" s="8">
+        <f>B32*0.124</f>
+        <v/>
+      </c>
+      <c r="D32" s="9">
+        <f>B32-C32</f>
+        <v/>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr"/>
-      <c r="G25" s="11" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="F32" s="10" t="inlineStr"/>
+      <c r="G32" s="11" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>Robe bustier Chiara Ferragni noire — M</t>
         </is>
       </c>
-      <c r="B26" s="15" t="n">
+      <c r="B33" s="13" t="n">
         <v>69</v>
       </c>
-      <c r="C26" s="16">
-        <f>B26*0.124</f>
-        <v/>
-      </c>
-      <c r="D26" s="17">
-        <f>B26-C26</f>
-        <v/>
-      </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="C33" s="14">
+        <f>B33*0.124</f>
+        <v/>
+      </c>
+      <c r="D33" s="15">
+        <f>B33-C33</f>
+        <v/>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="F26" s="18" t="inlineStr"/>
-      <c r="G26" s="19" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="F33" s="16" t="inlineStr"/>
+      <c r="G33" s="17" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>Ballerines Massimo Dutti cuir rouge — 40 IT</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n">
+      <c r="B34" s="7" t="n">
         <v>59</v>
       </c>
-      <c r="C27" s="8">
-        <f>B27*0.124</f>
-        <v/>
-      </c>
-      <c r="D27" s="9">
-        <f>B27-C27</f>
-        <v/>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="C34" s="8">
+        <f>B34*0.124</f>
+        <v/>
+      </c>
+      <c r="D34" s="9">
+        <f>B34-C34</f>
+        <v/>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
+      <c r="F34" s="10" t="inlineStr">
         <is>
           <t>Pas Vinted : article neuf</t>
         </is>
       </c>
-      <c r="G27" s="11" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="G34" s="11" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>Robe Pier Antonio Gaspari bleu marine — 42</t>
         </is>
       </c>
-      <c r="B28" s="15" t="n">
+      <c r="B35" s="13" t="n">
         <v>59</v>
       </c>
-      <c r="C28" s="16">
-        <f>B28*0.124</f>
-        <v/>
-      </c>
-      <c r="D28" s="17">
-        <f>B28-C28</f>
-        <v/>
-      </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="C35" s="14">
+        <f>B35*0.124</f>
+        <v/>
+      </c>
+      <c r="D35" s="15">
+        <f>B35-C35</f>
+        <v/>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="F28" s="18" t="inlineStr">
+      <c r="F35" s="16" t="inlineStr">
         <is>
           <t>Orthographe : Pier ANTONIO</t>
         </is>
       </c>
-      <c r="G28" s="19" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="G35" s="17" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Baskets Geox gris / argent — 35</t>
         </is>
       </c>
-      <c r="B29" s="7" t="n">
+      <c r="B36" s="7" t="n">
         <v>49</v>
       </c>
-      <c r="C29" s="8">
-        <f>B29*0.124</f>
-        <v/>
-      </c>
-      <c r="D29" s="9">
-        <f>B29-C29</f>
-        <v/>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="C36" s="8">
+        <f>B36*0.124</f>
+        <v/>
+      </c>
+      <c r="D36" s="9">
+        <f>B36-C36</f>
+        <v/>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F29" s="10" t="inlineStr"/>
-      <c r="G29" s="11" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="F36" s="10" t="inlineStr"/>
+      <c r="G36" s="11" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>Toupies Beyblade Hasbro — LOT de 4, n°1</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="n">
+        <v>49</v>
+      </c>
+      <c r="C37" s="14">
+        <f>B37*0.124</f>
+        <v/>
+      </c>
+      <c r="D37" s="15">
+        <f>B37-C37</f>
+        <v/>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>Leboncoin + Vinted</t>
+        </is>
+      </c>
+      <c r="F37" s="16" t="inlineStr">
+        <is>
+          <t>Rentrée scolaire : publier avant le 1er septembre</t>
+        </is>
+      </c>
+      <c r="G37" s="17" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Toupies Beyblade Hasbro — LOT de 4, n°2</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>49</v>
+      </c>
+      <c r="C38" s="8">
+        <f>B38*0.124</f>
+        <v/>
+      </c>
+      <c r="D38" s="9">
+        <f>B38-C38</f>
+        <v/>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Leboncoin + Vinted</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>À publier quand le 1er lot est vendu</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>Robby VP550W pompe immergée 550 W — 1ʳᵉ</t>
         </is>
       </c>
-      <c r="B30" s="15" t="n">
+      <c r="B39" s="13" t="n">
         <v>42</v>
       </c>
-      <c r="C30" s="16">
-        <f>B30*0.124</f>
-        <v/>
-      </c>
-      <c r="D30" s="17">
-        <f>B30-C30</f>
-        <v/>
-      </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="C39" s="14">
+        <f>B39*0.124</f>
+        <v/>
+      </c>
+      <c r="D39" s="15">
+        <f>B39-C39</f>
+        <v/>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Leboncoin, main propre</t>
         </is>
       </c>
-      <c r="F30" s="18" t="inlineStr">
+      <c r="F39" s="16" t="inlineStr">
         <is>
           <t>« Très bon état, jamais utilisée » · JAMAIS d'expédition</t>
         </is>
       </c>
-      <c r="G30" s="19" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="G39" s="17" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>Robby VP550W pompe immergée 550 W — 2ᵉ</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n">
+      <c r="B40" s="7" t="n">
         <v>42</v>
       </c>
-      <c r="C31" s="8">
-        <f>B31*0.124</f>
-        <v/>
-      </c>
-      <c r="D31" s="9">
-        <f>B31-C31</f>
-        <v/>
-      </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="C40" s="8">
+        <f>B40*0.124</f>
+        <v/>
+      </c>
+      <c r="D40" s="9">
+        <f>B40-C40</f>
+        <v/>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>Leboncoin, main propre</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="F40" s="10" t="inlineStr">
         <is>
           <t>À publier quand la 1ʳᵉ est vendue</t>
         </is>
       </c>
-      <c r="G31" s="11" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="14" t="inlineStr">
+      <c r="G40" s="11" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>Morgan — jean bleu clair T.40</t>
         </is>
       </c>
-      <c r="B32" s="15" t="n">
+      <c r="B41" s="13" t="n">
         <v>19</v>
       </c>
-      <c r="C32" s="16">
-        <f>B32*0.124</f>
-        <v/>
-      </c>
-      <c r="D32" s="17">
-        <f>B32-C32</f>
-        <v/>
-      </c>
-      <c r="E32" s="14" t="inlineStr">
+      <c r="C41" s="14">
+        <f>B41*0.124</f>
+        <v/>
+      </c>
+      <c r="D41" s="15">
+        <f>B41-C41</f>
+        <v/>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F32" s="18" t="inlineStr"/>
-      <c r="G32" s="19" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="F41" s="16" t="inlineStr"/>
+      <c r="G41" s="17" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>Morgan — jupe marron</t>
         </is>
       </c>
-      <c r="B33" s="7" t="n">
+      <c r="B42" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="C33" s="8">
-        <f>B33*0.124</f>
-        <v/>
-      </c>
-      <c r="D33" s="9">
-        <f>B33-C33</f>
-        <v/>
-      </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="C42" s="8">
+        <f>B42*0.124</f>
+        <v/>
+      </c>
+      <c r="D42" s="9">
+        <f>B42-C42</f>
+        <v/>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F33" s="10" t="inlineStr"/>
-      <c r="G33" s="11" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="14" t="inlineStr">
+      <c r="F42" s="10" t="inlineStr"/>
+      <c r="G42" s="11" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>Morgan — pantalon blanc T.40</t>
         </is>
       </c>
-      <c r="B34" s="15" t="n">
+      <c r="B43" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="C34" s="16">
-        <f>B34*0.124</f>
-        <v/>
-      </c>
-      <c r="D34" s="17">
-        <f>B34-C34</f>
-        <v/>
-      </c>
-      <c r="E34" s="14" t="inlineStr">
+      <c r="C43" s="14">
+        <f>B43*0.124</f>
+        <v/>
+      </c>
+      <c r="D43" s="15">
+        <f>B43-C43</f>
+        <v/>
+      </c>
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F34" s="18" t="inlineStr"/>
-      <c r="G34" s="19" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="F43" s="16" t="inlineStr"/>
+      <c r="G43" s="17" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>Morgan — polo rouge à écusson doré L</t>
         </is>
       </c>
-      <c r="B35" s="7" t="n">
+      <c r="B44" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="C35" s="8">
-        <f>B35*0.124</f>
-        <v/>
-      </c>
-      <c r="D35" s="9">
-        <f>B35-C35</f>
-        <v/>
-      </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="C44" s="8">
+        <f>B44*0.124</f>
+        <v/>
+      </c>
+      <c r="D44" s="9">
+        <f>B44-C44</f>
+        <v/>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F35" s="10" t="inlineStr"/>
-      <c r="G35" s="11" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="14" t="inlineStr">
+      <c r="F44" s="10" t="inlineStr"/>
+      <c r="G44" s="11" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
         <is>
           <t>Morgan — top camel lurex L</t>
         </is>
       </c>
-      <c r="B36" s="15" t="n">
+      <c r="B45" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="C36" s="16">
-        <f>B36*0.124</f>
-        <v/>
-      </c>
-      <c r="D36" s="17">
-        <f>B36-C36</f>
-        <v/>
-      </c>
-      <c r="E36" s="14" t="inlineStr">
+      <c r="C45" s="14">
+        <f>B45*0.124</f>
+        <v/>
+      </c>
+      <c r="D45" s="15">
+        <f>B45-C45</f>
+        <v/>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F36" s="18" t="inlineStr"/>
-      <c r="G36" s="19" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+      <c r="F45" s="16" t="inlineStr"/>
+      <c r="G45" s="17" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>Morgan — polo blanc L</t>
         </is>
       </c>
-      <c r="B37" s="7" t="n">
+      <c r="B46" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="C37" s="8">
-        <f>B37*0.124</f>
-        <v/>
-      </c>
-      <c r="D37" s="9">
-        <f>B37-C37</f>
-        <v/>
-      </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="C46" s="8">
+        <f>B46*0.124</f>
+        <v/>
+      </c>
+      <c r="D46" s="9">
+        <f>B46-C46</f>
+        <v/>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F37" s="10" t="inlineStr"/>
-      <c r="G37" s="11" t="n"/>
-    </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="22" t="inlineStr">
+      <c r="F46" s="10" t="inlineStr"/>
+      <c r="G46" s="11" t="n"/>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>3. LIQUIDER — vendre pour récupérer la trésorerie, pas pour la marge</t>
         </is>
       </c>
-      <c r="B38" s="23" t="n"/>
-      <c r="C38" s="23" t="n"/>
-      <c r="D38" s="23" t="n"/>
-      <c r="E38" s="23" t="n"/>
-      <c r="F38" s="23" t="n"/>
-      <c r="G38" s="23" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="B47" s="23" t="n"/>
+      <c r="C47" s="23" t="n"/>
+      <c r="D47" s="23" t="n"/>
+      <c r="E47" s="23" t="n"/>
+      <c r="F47" s="23" t="n"/>
+      <c r="G47" s="23" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>New Balance GS 1906 Alkaline Green — 38½</t>
         </is>
       </c>
-      <c r="B39" s="7" t="n">
+      <c r="B48" s="7" t="n">
         <v>99</v>
       </c>
-      <c r="C39" s="8">
-        <f>B39*0.124</f>
-        <v/>
-      </c>
-      <c r="D39" s="9">
-        <f>B39-C39</f>
-        <v/>
-      </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="C48" s="8">
+        <f>B48*0.124</f>
+        <v/>
+      </c>
+      <c r="D48" s="9">
+        <f>B48-C48</f>
+        <v/>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="F39" s="10" t="inlineStr">
+      <c r="F48" s="10" t="inlineStr">
         <is>
           <t>Préciser « modèle GS », réf. G19064IK</t>
         </is>
       </c>
-      <c r="G39" s="11" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="14" t="inlineStr">
+      <c r="G48" s="11" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t>Baskets Emporio Armani bleu lavande — 36</t>
         </is>
       </c>
-      <c r="B40" s="15" t="n">
+      <c r="B49" s="13" t="n">
         <v>69</v>
       </c>
-      <c r="C40" s="16">
-        <f>B40*0.124</f>
-        <v/>
-      </c>
-      <c r="D40" s="17">
-        <f>B40-C40</f>
-        <v/>
-      </c>
-      <c r="E40" s="14" t="inlineStr">
+      <c r="C49" s="14">
+        <f>B49*0.124</f>
+        <v/>
+      </c>
+      <c r="D49" s="15">
+        <f>B49-C49</f>
+        <v/>
+      </c>
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="F40" s="18" t="inlineStr"/>
-      <c r="G40" s="19" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
+      <c r="F49" s="16" t="inlineStr"/>
+      <c r="G49" s="17" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>Tommy Jeans baskets basses noir / blanc — 40</t>
         </is>
       </c>
-      <c r="B41" s="7" t="n">
+      <c r="B50" s="7" t="n">
         <v>65</v>
       </c>
-      <c r="C41" s="8">
-        <f>B41*0.124</f>
-        <v/>
-      </c>
-      <c r="D41" s="9">
-        <f>B41-C41</f>
-        <v/>
-      </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="C50" s="8">
+        <f>B50*0.124</f>
+        <v/>
+      </c>
+      <c r="D50" s="9">
+        <f>B50-C50</f>
+        <v/>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F41" s="10" t="inlineStr"/>
-      <c r="G41" s="11" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="14" t="inlineStr">
+      <c r="F50" s="10" t="inlineStr"/>
+      <c r="G50" s="11" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t>New Balance 650 blanche montante — 44</t>
         </is>
       </c>
-      <c r="B42" s="15" t="n">
+      <c r="B51" s="13" t="n">
         <v>65</v>
       </c>
-      <c r="C42" s="16">
-        <f>B42*0.124</f>
-        <v/>
-      </c>
-      <c r="D42" s="17">
-        <f>B42-C42</f>
-        <v/>
-      </c>
-      <c r="E42" s="14" t="inlineStr">
+      <c r="C51" s="14">
+        <f>B51*0.124</f>
+        <v/>
+      </c>
+      <c r="D51" s="15">
+        <f>B51-C51</f>
+        <v/>
+      </c>
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="F42" s="18" t="inlineStr"/>
-      <c r="G42" s="19" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
+      <c r="F51" s="16" t="inlineStr"/>
+      <c r="G51" s="17" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>New Balance BB80 blanc / marine — 38</t>
         </is>
       </c>
-      <c r="B43" s="7" t="n">
+      <c r="B52" s="7" t="n">
         <v>54</v>
       </c>
-      <c r="C43" s="8">
-        <f>B43*0.124</f>
-        <v/>
-      </c>
-      <c r="D43" s="9">
-        <f>B43-C43</f>
-        <v/>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="C52" s="8">
+        <f>B52*0.124</f>
+        <v/>
+      </c>
+      <c r="D52" s="9">
+        <f>B52-C52</f>
+        <v/>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="F43" s="10" t="inlineStr"/>
-      <c r="G43" s="11" t="n"/>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="24" t="inlineStr">
+      <c r="F52" s="10" t="inlineStr"/>
+      <c r="G52" s="11" t="n"/>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="22" t="inlineStr">
+        <is>
+          <t>5. POKÉMON — import du Japon, marges minces, vérifier le marché avant de publier</t>
+        </is>
+      </c>
+      <c r="B53" s="23" t="n"/>
+      <c r="C53" s="23" t="n"/>
+      <c r="D53" s="23" t="n"/>
+      <c r="E53" s="23" t="n"/>
+      <c r="F53" s="23" t="n"/>
+      <c r="G53" s="23" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Boosters Nihil Zero M3 — LOT de 5, n°1</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="C54" s="8">
+        <f>B54*0.124</f>
+        <v/>
+      </c>
+      <c r="D54" s="9">
+        <f>B54-C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>Leboncoin, main propre</t>
+        </is>
+      </c>
+      <c r="F54" s="10" t="inlineStr">
+        <is>
+          <t>3,40 €/booster · le moins cher du net est à 3,50 € (Pikastore)</t>
+        </is>
+      </c>
+      <c r="G54" s="11" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t>Boosters Nihil Zero M3 — LOT de 5, n°2</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C55" s="14">
+        <f>B55*0.124</f>
+        <v/>
+      </c>
+      <c r="D55" s="15">
+        <f>B55-C55</f>
+        <v/>
+      </c>
+      <c r="E55" s="12" t="inlineStr">
+        <is>
+          <t>Leboncoin, main propre</t>
+        </is>
+      </c>
+      <c r="F55" s="16" t="inlineStr">
+        <is>
+          <t>À publier quand le n°1 est vendu</t>
+        </is>
+      </c>
+      <c r="G55" s="17" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>Boosters Nihil Zero M3 — LOT de 5, n°3</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="C56" s="8">
+        <f>B56*0.124</f>
+        <v/>
+      </c>
+      <c r="D56" s="9">
+        <f>B56-C56</f>
+        <v/>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>Leboncoin, main propre</t>
+        </is>
+      </c>
+      <c r="F56" s="10" t="inlineStr">
+        <is>
+          <t>À publier quand le n°2 est vendu</t>
+        </is>
+      </c>
+      <c r="G56" s="11" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>Boosters Nihil Zero M3 — LOT de 5, n°4</t>
+        </is>
+      </c>
+      <c r="B57" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C57" s="14">
+        <f>B57*0.124</f>
+        <v/>
+      </c>
+      <c r="D57" s="15">
+        <f>B57-C57</f>
+        <v/>
+      </c>
+      <c r="E57" s="12" t="inlineStr">
+        <is>
+          <t>Leboncoin, main propre</t>
+        </is>
+      </c>
+      <c r="F57" s="16" t="inlineStr">
+        <is>
+          <t>À publier quand le n°3 est vendu</t>
+        </is>
+      </c>
+      <c r="G57" s="17" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Boosters Nihil Zero M3 — LOT de 5, n°5</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="C58" s="8">
+        <f>B58*0.124</f>
+        <v/>
+      </c>
+      <c r="D58" s="9">
+        <f>B58-C58</f>
+        <v/>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Leboncoin, main propre</t>
+        </is>
+      </c>
+      <c r="F58" s="10" t="inlineStr">
+        <is>
+          <t>À publier quand le n°4 est vendu</t>
+        </is>
+      </c>
+      <c r="G58" s="11" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>Boosters Nihil Zero M3 — LOT de 5, n°6</t>
+        </is>
+      </c>
+      <c r="B59" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C59" s="14">
+        <f>B59*0.124</f>
+        <v/>
+      </c>
+      <c r="D59" s="15">
+        <f>B59-C59</f>
+        <v/>
+      </c>
+      <c r="E59" s="12" t="inlineStr">
+        <is>
+          <t>Leboncoin, main propre</t>
+        </is>
+      </c>
+      <c r="F59" s="16" t="inlineStr">
+        <is>
+          <t>À publier quand le n°5 est vendu</t>
+        </is>
+      </c>
+      <c r="G59" s="17" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Booster High Class MEGA Dream ex M2a — à l'unité</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C60" s="8">
+        <f>B60*0.124</f>
+        <v/>
+      </c>
+      <c r="D60" s="9">
+        <f>B60-C60</f>
+        <v/>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>Leboncoin, main propre</t>
+        </is>
+      </c>
+      <c r="F60" s="10" t="inlineStr">
+        <is>
+          <t>SEUIL 14,78 € · vérifier le prix du booster seul avant de publier</t>
+        </is>
+      </c>
+      <c r="G60" s="11" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>Boosters MEGA Storm Emeralda M6 — LOT de 2</t>
+        </is>
+      </c>
+      <c r="B61" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C61" s="14">
+        <f>B61*0.124</f>
+        <v/>
+      </c>
+      <c r="D61" s="15">
+        <f>B61-C61</f>
+        <v/>
+      </c>
+      <c r="E61" s="12" t="inlineStr">
+        <is>
+          <t>Leboncoin, main propre</t>
+        </is>
+      </c>
+      <c r="F61" s="16" t="inlineStr">
+        <is>
+          <t>SEUIL 14,54 € · set sorti le 31/07/2026, forte demande</t>
+        </is>
+      </c>
+      <c r="G61" s="17" t="n"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="24" t="inlineStr">
         <is>
           <t>4. PLUS TARD — ne pas publier maintenant</t>
         </is>
       </c>
-      <c r="B44" s="25" t="n"/>
-      <c r="C44" s="25" t="n"/>
-      <c r="D44" s="25" t="n"/>
-      <c r="E44" s="25" t="n"/>
-      <c r="F44" s="25" t="n"/>
-      <c r="G44" s="25" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
+      <c r="B62" s="25" t="n"/>
+      <c r="C62" s="25" t="n"/>
+      <c r="D62" s="25" t="n"/>
+      <c r="E62" s="25" t="n"/>
+      <c r="F62" s="25" t="n"/>
+      <c r="G62" s="25" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>Lot 20 sandales et tongs — EN LOT</t>
         </is>
       </c>
-      <c r="B45" s="7" t="n">
+      <c r="B63" s="7" t="n">
         <v>199</v>
       </c>
-      <c r="C45" s="8">
-        <f>B45*0.124</f>
-        <v/>
-      </c>
-      <c r="D45" s="9">
-        <f>B45-C45</f>
-        <v/>
-      </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="C63" s="8">
+        <f>B63*0.124</f>
+        <v/>
+      </c>
+      <c r="D63" s="9">
+        <f>B63-C63</f>
+        <v/>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
         <is>
           <t>Leboncoin B2B</t>
         </is>
       </c>
-      <c r="F45" s="10" t="inlineStr">
+      <c r="F63" s="10" t="inlineStr">
         <is>
           <t>FÉVRIER-MARS, quand le revendeur prépare l'été</t>
         </is>
       </c>
-      <c r="G45" s="11" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="14" t="inlineStr">
+      <c r="G63" s="11" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
         <is>
           <t>Adidas Yeezy 700 V3 Mono Safflower — 38</t>
         </is>
       </c>
-      <c r="B46" s="26" t="inlineStr">
+      <c r="B64" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C46" s="26" t="inlineStr">
+      <c r="C64" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D46" s="26" t="inlineStr">
+      <c r="D64" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E46" s="14" t="inlineStr">
+      <c r="E64" s="12" t="inlineStr">
         <is>
           <t>Vinted</t>
         </is>
       </c>
-      <c r="F46" s="18" t="inlineStr">
+      <c r="F64" s="16" t="inlineStr">
         <is>
           <t>BLOQUÉ : authentification requise avant de fixer le prix</t>
         </is>
       </c>
-      <c r="G46" s="19" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="27" t="inlineStr">
+      <c r="G64" s="17" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="27" t="inlineStr">
         <is>
           <t>TOTAL — 36 annonces chiffrées</t>
         </is>
       </c>
-      <c r="B47" s="28">
-        <f>B6+B8+B9+B10+B11+B12+B13+B15+B16+B17+B18+B19+B20+B21+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36+B37+B39+B40+B41+B42+B43+B45</f>
-        <v/>
-      </c>
-      <c r="C47" s="29">
-        <f>B47*0.124</f>
-        <v/>
-      </c>
-      <c r="D47" s="28">
-        <f>B47-C47</f>
-        <v/>
-      </c>
-      <c r="E47" s="30" t="n"/>
-      <c r="F47" s="30" t="n"/>
-      <c r="G47" s="30" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="B65" s="28">
+        <f>B6+B7+B8+B9+B10+B11+B12+B13+B15+B16+B17+B18+B19+B20+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36+B37+B38+B39+B40+B41+B42+B43+B44+B45+B46+B48+B49+B50+B51+B52+B54+B55+B56+B57+B58+B59+B60+B61+B63</f>
+        <v/>
+      </c>
+      <c r="C65" s="29">
+        <f>B65*0.124</f>
+        <v/>
+      </c>
+      <c r="D65" s="28">
+        <f>B65-C65</f>
+        <v/>
+      </c>
+      <c r="E65" s="30" t="n"/>
+      <c r="F65" s="30" t="n"/>
+      <c r="G65" s="30" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>Le prix de la Yeezy sera fixé après authentification (10-20 €).</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>Règle : ces prix sont déjà calés sous le moins cher trouvé sur Internet. Ne pas les remonter.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>URSSAF = 12,3 % de cotisations + 0,1 % de CFP, calculé sur le prix de vente encaissé. À mettre de côté à chaque vente, pas à la fin du trimestre.</t>
         </is>

</xml_diff>

<commit_message>
regle des deux tiers: le High Class passe en bundle, invendable seul
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -2049,11 +2049,11 @@
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>Boosters Nihil Zero M3 — LOT de 5, n°6</t>
+          <t>BUNDLE : High Class MEGA Dream ex + 5 Nihil Zero</t>
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="C59" s="14">
         <f>B59*0.124</f>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>À publier quand le n°5 est vendu</t>
+          <t>Le High Class est INVENDABLE SEUL : marché 12,99 €, coût 12,95 €</t>
         </is>
       </c>
       <c r="G59" s="17" t="n"/>
@@ -2078,11 +2078,11 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>Booster High Class MEGA Dream ex M2a — à l'unité</t>
+          <t>Boosters MEGA Storm Emeralda M6 — LOT de 2</t>
         </is>
       </c>
       <c r="B60" s="7" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C60" s="8">
         <f>B60*0.124</f>
@@ -2099,153 +2099,124 @@
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t>SEUIL 14,78 € · vérifier le prix du booster seul avant de publier</t>
+          <t>SEUIL 14,54 € · set sorti le 31/07/2026, forte demande</t>
         </is>
       </c>
       <c r="G60" s="11" t="n"/>
     </row>
-    <row r="61">
-      <c r="A61" s="12" t="inlineStr">
-        <is>
-          <t>Boosters MEGA Storm Emeralda M6 — LOT de 2</t>
-        </is>
-      </c>
-      <c r="B61" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="C61" s="14">
-        <f>B61*0.124</f>
-        <v/>
-      </c>
-      <c r="D61" s="15">
-        <f>B61-C61</f>
-        <v/>
-      </c>
-      <c r="E61" s="12" t="inlineStr">
-        <is>
-          <t>Leboncoin, main propre</t>
-        </is>
-      </c>
-      <c r="F61" s="16" t="inlineStr">
-        <is>
-          <t>SEUIL 14,54 € · set sorti le 31/07/2026, forte demande</t>
-        </is>
-      </c>
-      <c r="G61" s="17" t="n"/>
-    </row>
-    <row r="62" ht="22" customHeight="1">
-      <c r="A62" s="24" t="inlineStr">
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="24" t="inlineStr">
         <is>
           <t>4. PLUS TARD — ne pas publier maintenant</t>
         </is>
       </c>
-      <c r="B62" s="25" t="n"/>
-      <c r="C62" s="25" t="n"/>
-      <c r="D62" s="25" t="n"/>
-      <c r="E62" s="25" t="n"/>
-      <c r="F62" s="25" t="n"/>
-      <c r="G62" s="25" t="n"/>
+      <c r="B61" s="25" t="n"/>
+      <c r="C61" s="25" t="n"/>
+      <c r="D61" s="25" t="n"/>
+      <c r="E61" s="25" t="n"/>
+      <c r="F61" s="25" t="n"/>
+      <c r="G61" s="25" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Lot 20 sandales et tongs — EN LOT</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="n">
+        <v>199</v>
+      </c>
+      <c r="C62" s="8">
+        <f>B62*0.124</f>
+        <v/>
+      </c>
+      <c r="D62" s="9">
+        <f>B62-C62</f>
+        <v/>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>Leboncoin B2B</t>
+        </is>
+      </c>
+      <c r="F62" s="10" t="inlineStr">
+        <is>
+          <t>FÉVRIER-MARS, quand le revendeur prépare l'été</t>
+        </is>
+      </c>
+      <c r="G62" s="11" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t>Lot 20 sandales et tongs — EN LOT</t>
-        </is>
-      </c>
-      <c r="B63" s="7" t="n">
-        <v>199</v>
-      </c>
-      <c r="C63" s="8">
-        <f>B63*0.124</f>
-        <v/>
-      </c>
-      <c r="D63" s="9">
-        <f>B63-C63</f>
-        <v/>
-      </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>Leboncoin B2B</t>
-        </is>
-      </c>
-      <c r="F63" s="10" t="inlineStr">
-        <is>
-          <t>FÉVRIER-MARS, quand le revendeur prépare l'été</t>
-        </is>
-      </c>
-      <c r="G63" s="11" t="n"/>
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>Adidas Yeezy 700 V3 Mono Safflower — 38</t>
+        </is>
+      </c>
+      <c r="B63" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C63" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D63" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E63" s="12" t="inlineStr">
+        <is>
+          <t>Vinted</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>BLOQUÉ : authentification requise avant de fixer le prix</t>
+        </is>
+      </c>
+      <c r="G63" s="17" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="12" t="inlineStr">
-        <is>
-          <t>Adidas Yeezy 700 V3 Mono Safflower — 38</t>
-        </is>
-      </c>
-      <c r="B64" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C64" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D64" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E64" s="12" t="inlineStr">
-        <is>
-          <t>Vinted</t>
-        </is>
-      </c>
-      <c r="F64" s="16" t="inlineStr">
-        <is>
-          <t>BLOQUÉ : authentification requise avant de fixer le prix</t>
-        </is>
-      </c>
-      <c r="G64" s="17" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="27" t="inlineStr">
+      <c r="A64" s="27" t="inlineStr">
         <is>
           <t>TOTAL — 36 annonces chiffrées</t>
         </is>
       </c>
-      <c r="B65" s="28">
-        <f>B6+B7+B8+B9+B10+B11+B12+B13+B15+B16+B17+B18+B19+B20+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36+B37+B38+B39+B40+B41+B42+B43+B44+B45+B46+B48+B49+B50+B51+B52+B54+B55+B56+B57+B58+B59+B60+B61+B63</f>
-        <v/>
-      </c>
-      <c r="C65" s="29">
-        <f>B65*0.124</f>
-        <v/>
-      </c>
-      <c r="D65" s="28">
-        <f>B65-C65</f>
-        <v/>
-      </c>
-      <c r="E65" s="30" t="n"/>
-      <c r="F65" s="30" t="n"/>
-      <c r="G65" s="30" t="n"/>
+      <c r="B64" s="28">
+        <f>B6+B7+B8+B9+B10+B11+B12+B13+B15+B16+B17+B18+B19+B20+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36+B37+B38+B39+B40+B41+B42+B43+B44+B45+B46+B48+B49+B50+B51+B52+B54+B55+B56+B57+B58+B59+B60+B62</f>
+        <v/>
+      </c>
+      <c r="C64" s="29">
+        <f>B64*0.124</f>
+        <v/>
+      </c>
+      <c r="D64" s="28">
+        <f>B64-C64</f>
+        <v/>
+      </c>
+      <c r="E64" s="30" t="n"/>
+      <c r="F64" s="30" t="n"/>
+      <c r="G64" s="30" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Le prix de la Yeezy sera fixé après authentification (10-20 €).</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Le prix de la Yeezy sera fixé après authentification (10-20 €).</t>
+          <t>Règle : ces prix sont déjà calés sous le moins cher trouvé sur Internet. Ne pas les remonter.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>Règle : ces prix sont déjà calés sous le moins cher trouvé sur Internet. Ne pas les remonter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>URSSAF = 12,3 % de cotisations + 0,1 % de CFP, calculé sur le prix de vente encaissé. À mettre de côté à chaque vente, pas à la fin du trimestre.</t>
         </is>

</xml_diff>

<commit_message>
pompes Robby: bordereau ERA integre, trois lots distincts, deux defauts declares
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -1541,11 +1541,11 @@
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>Robby VP550W pompe immergée 550 W — 1ʳᵉ</t>
+          <t>Robby VP550W pompe immergée — ligne 84, occasion</t>
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C39" s="14">
         <f>B39*0.124</f>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>« Très bon état, jamais utilisée » · JAMAIS d'expédition</t>
+          <t>Tester avant de publier · JAMAIS d'expédition, 4,8 kg</t>
         </is>
       </c>
       <c r="G39" s="17" t="n"/>
@@ -1570,11 +1570,11 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Robby VP550W pompe immergée 550 W — 2ᵉ</t>
+          <t>Robby VP550W pompe immergée — ligne 122, SOCLE CASSÉ</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C40" s="8">
         <f>B40*0.124</f>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t>À publier quand la 1ʳᵉ est vendue</t>
+          <t>DÉFAUT À DÉCLARER + photo du socle · JAMAIS d'expédition</t>
         </is>
       </c>
       <c r="G40" s="11" t="n"/>

</xml_diff>

<commit_message>
pokemon: booster High Class preleve pour usage personnel
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -2049,11 +2049,11 @@
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>BUNDLE : High Class MEGA Dream ex + 5 Nihil Zero</t>
+          <t>Boosters Nihil Zero M3 — LOT de 5, n°6</t>
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="C59" s="14">
         <f>B59*0.124</f>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>Le High Class est INVENDABLE SEUL : marché 12,99 €, coût 12,95 €</t>
+          <t>À publier quand le n°5 est vendu</t>
         </is>
       </c>
       <c r="G59" s="17" t="n"/>

</xml_diff>

<commit_message>
box Nihil Zero scellee: deux lots de 15 au lieu de six lots de cinq
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1891,7 +1891,7 @@
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="22" t="inlineStr">
         <is>
-          <t>5. POKÉMON — import du Japon, marges minces, vérifier le marché avant de publier</t>
+          <t>5. POKÉMON — import du Japon, marges minces</t>
         </is>
       </c>
       <c r="B53" s="23" t="n"/>
@@ -1904,11 +1904,11 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>Boosters Nihil Zero M3 — LOT de 5, n°1</t>
+          <t>Boosters Nihil Zero M3 — LOT de 15, n°1</t>
         </is>
       </c>
       <c r="B54" s="7" t="n">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="C54" s="8">
         <f>B54*0.124</f>
@@ -1925,7 +1925,7 @@
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t>3,40 €/booster · le moins cher du net est à 3,50 € (Pikastore)</t>
+          <t>PHOTOGRAPHIER LE BLISTER SCELLÉ avant d'ouvrir la box</t>
         </is>
       </c>
       <c r="G54" s="11" t="n"/>
@@ -1933,11 +1933,11 @@
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>Boosters Nihil Zero M3 — LOT de 5, n°2</t>
+          <t>Boosters Nihil Zero M3 — LOT de 15, n°2</t>
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="C55" s="14">
         <f>B55*0.124</f>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
-          <t>À publier quand le n°1 est vendu</t>
+          <t>« Boosters non pesés, non triés » dans l'annonce</t>
         </is>
       </c>
       <c r="G55" s="17" t="n"/>
@@ -1962,11 +1962,11 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>Boosters Nihil Zero M3 — LOT de 5, n°3</t>
+          <t>Boosters MEGA Storm Emeralda M6 — LOT de 2</t>
         </is>
       </c>
       <c r="B56" s="7" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C56" s="8">
         <f>B56*0.124</f>
@@ -1983,48 +1983,32 @@
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t>À publier quand le n°2 est vendu</t>
+          <t>SEUIL 14,54 € · set sorti le 31/07/2026, forte demande</t>
         </is>
       </c>
       <c r="G56" s="11" t="n"/>
     </row>
-    <row r="57">
-      <c r="A57" s="12" t="inlineStr">
-        <is>
-          <t>Boosters Nihil Zero M3 — LOT de 5, n°4</t>
-        </is>
-      </c>
-      <c r="B57" s="13" t="n">
-        <v>17</v>
-      </c>
-      <c r="C57" s="14">
-        <f>B57*0.124</f>
-        <v/>
-      </c>
-      <c r="D57" s="15">
-        <f>B57-C57</f>
-        <v/>
-      </c>
-      <c r="E57" s="12" t="inlineStr">
-        <is>
-          <t>Leboncoin, main propre</t>
-        </is>
-      </c>
-      <c r="F57" s="16" t="inlineStr">
-        <is>
-          <t>À publier quand le n°3 est vendu</t>
-        </is>
-      </c>
-      <c r="G57" s="17" t="n"/>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="24" t="inlineStr">
+        <is>
+          <t>4. PLUS TARD — ne pas publier maintenant</t>
+        </is>
+      </c>
+      <c r="B57" s="25" t="n"/>
+      <c r="C57" s="25" t="n"/>
+      <c r="D57" s="25" t="n"/>
+      <c r="E57" s="25" t="n"/>
+      <c r="F57" s="25" t="n"/>
+      <c r="G57" s="25" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>Boosters Nihil Zero M3 — LOT de 5, n°5</t>
+          <t>Lot 20 sandales et tongs — EN LOT</t>
         </is>
       </c>
       <c r="B58" s="7" t="n">
-        <v>17</v>
+        <v>199</v>
       </c>
       <c r="C58" s="8">
         <f>B58*0.124</f>
@@ -2036,12 +2020,12 @@
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin, main propre</t>
+          <t>Leboncoin B2B</t>
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t>À publier quand le n°4 est vendu</t>
+          <t>FÉVRIER-MARS, quand le revendeur prépare l'été</t>
         </is>
       </c>
       <c r="G58" s="11" t="n"/>
@@ -2049,174 +2033,74 @@
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>Boosters Nihil Zero M3 — LOT de 5, n°6</t>
-        </is>
-      </c>
-      <c r="B59" s="13" t="n">
-        <v>17</v>
-      </c>
-      <c r="C59" s="14">
-        <f>B59*0.124</f>
-        <v/>
-      </c>
-      <c r="D59" s="15">
-        <f>B59-C59</f>
-        <v/>
+          <t>Adidas Yeezy 700 V3 Mono Safflower — 38</t>
+        </is>
+      </c>
+      <c r="B59" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C59" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D59" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="E59" s="12" t="inlineStr">
         <is>
-          <t>Leboncoin, main propre</t>
+          <t>Vinted</t>
         </is>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>À publier quand le n°5 est vendu</t>
+          <t>BLOQUÉ : authentification requise avant de fixer le prix</t>
         </is>
       </c>
       <c r="G59" s="17" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>Boosters MEGA Storm Emeralda M6 — LOT de 2</t>
-        </is>
-      </c>
-      <c r="B60" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="C60" s="8">
+      <c r="A60" s="27" t="inlineStr">
+        <is>
+          <t>TOTAL — 36 annonces chiffrées</t>
+        </is>
+      </c>
+      <c r="B60" s="28">
+        <f>B6+B7+B8+B9+B10+B11+B12+B13+B15+B16+B17+B18+B19+B20+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36+B37+B38+B39+B40+B41+B42+B43+B44+B45+B46+B48+B49+B50+B51+B52+B54+B55+B56+B58</f>
+        <v/>
+      </c>
+      <c r="C60" s="29">
         <f>B60*0.124</f>
         <v/>
       </c>
-      <c r="D60" s="9">
+      <c r="D60" s="28">
         <f>B60-C60</f>
         <v/>
       </c>
-      <c r="E60" s="6" t="inlineStr">
-        <is>
-          <t>Leboncoin, main propre</t>
-        </is>
-      </c>
-      <c r="F60" s="10" t="inlineStr">
-        <is>
-          <t>SEUIL 14,54 € · set sorti le 31/07/2026, forte demande</t>
-        </is>
-      </c>
-      <c r="G60" s="11" t="n"/>
-    </row>
-    <row r="61" ht="22" customHeight="1">
-      <c r="A61" s="24" t="inlineStr">
-        <is>
-          <t>4. PLUS TARD — ne pas publier maintenant</t>
-        </is>
-      </c>
-      <c r="B61" s="25" t="n"/>
-      <c r="C61" s="25" t="n"/>
-      <c r="D61" s="25" t="n"/>
-      <c r="E61" s="25" t="n"/>
-      <c r="F61" s="25" t="n"/>
-      <c r="G61" s="25" t="n"/>
+      <c r="E60" s="30" t="n"/>
+      <c r="F60" s="30" t="n"/>
+      <c r="G60" s="30" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>Lot 20 sandales et tongs — EN LOT</t>
-        </is>
-      </c>
-      <c r="B62" s="7" t="n">
-        <v>199</v>
-      </c>
-      <c r="C62" s="8">
-        <f>B62*0.124</f>
-        <v/>
-      </c>
-      <c r="D62" s="9">
-        <f>B62-C62</f>
-        <v/>
-      </c>
-      <c r="E62" s="6" t="inlineStr">
-        <is>
-          <t>Leboncoin B2B</t>
-        </is>
-      </c>
-      <c r="F62" s="10" t="inlineStr">
-        <is>
-          <t>FÉVRIER-MARS, quand le revendeur prépare l'été</t>
-        </is>
-      </c>
-      <c r="G62" s="11" t="n"/>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Le prix de la Yeezy sera fixé après authentification (10-20 €).</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="12" t="inlineStr">
-        <is>
-          <t>Adidas Yeezy 700 V3 Mono Safflower — 38</t>
-        </is>
-      </c>
-      <c r="B63" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C63" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D63" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E63" s="12" t="inlineStr">
-        <is>
-          <t>Vinted</t>
-        </is>
-      </c>
-      <c r="F63" s="16" t="inlineStr">
-        <is>
-          <t>BLOQUÉ : authentification requise avant de fixer le prix</t>
-        </is>
-      </c>
-      <c r="G63" s="17" t="n"/>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Règle : ces prix sont déjà calés sous le moins cher trouvé sur Internet. Ne pas les remonter.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="27" t="inlineStr">
-        <is>
-          <t>TOTAL — 36 annonces chiffrées</t>
-        </is>
-      </c>
-      <c r="B64" s="28">
-        <f>B6+B7+B8+B9+B10+B11+B12+B13+B15+B16+B17+B18+B19+B20+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36+B37+B38+B39+B40+B41+B42+B43+B44+B45+B46+B48+B49+B50+B51+B52+B54+B55+B56+B57+B58+B59+B60+B62</f>
-        <v/>
-      </c>
-      <c r="C64" s="29">
-        <f>B64*0.124</f>
-        <v/>
-      </c>
-      <c r="D64" s="28">
-        <f>B64-C64</f>
-        <v/>
-      </c>
-      <c r="E64" s="30" t="n"/>
-      <c r="F64" s="30" t="n"/>
-      <c r="G64" s="30" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>Le prix de la Yeezy sera fixé après authentification (10-20 €).</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>Règle : ces prix sont déjà calés sous le moins cher trouvé sur Internet. Ne pas les remonter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>URSSAF = 12,3 % de cotisations + 0,1 % de CFP, calculé sur le prix de vente encaissé. À mettre de côté à chaque vente, pas à la fin du trimestre.</t>
         </is>

</xml_diff>

<commit_message>
beyblade: les deux lots distingues, ecart de cout documente
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -1487,7 +1487,7 @@
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>Toupies Beyblade Hasbro — LOT de 4, n°1</t>
+          <t>Toupies Beyblade Hasbro — LOT de 4, lot n°159</t>
         </is>
       </c>
       <c r="B37" s="13" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>Rentrée scolaire : publier avant le 1er septembre</t>
+          <t>Coût 21,54 € · marge 21,39 € · publier avant le 1er septembre</t>
         </is>
       </c>
       <c r="G37" s="17" t="n"/>
@@ -1516,7 +1516,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Toupies Beyblade Hasbro — LOT de 4, n°2</t>
+          <t>Toupies Beyblade Hasbro — LOT de 4, lot n°299</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t>À publier quand le 1er lot est vendu</t>
+          <t>Coût 40,71 € · marge 2,22 € seulement · à publier après le n°159</t>
         </is>
       </c>
       <c r="G38" s="11" t="n"/>

</xml_diff>

<commit_message>
hogan: nettoyees, annonce sans les traces d'essayage
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -1348,7 +1348,11 @@
           <t>Boutique</t>
         </is>
       </c>
-      <c r="F31" s="16" t="inlineStr"/>
+      <c r="F31" s="16" t="inlineStr">
+        <is>
+          <t>Nettoyées : « aucune trace visible », PAS « neuves » — 12 mois de garantie au lieu de 24</t>
+        </is>
+      </c>
       <c r="G31" s="17" t="n"/>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
morgan: six annonces a l'unite, deux prix remontes au plancher
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C45" s="14">
         <f>B45*0.124</f>
@@ -1726,7 +1726,11 @@
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F45" s="16" t="inlineStr"/>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>Remonté de 12 à 15 € : 12 € passait sous le plancher</t>
+        </is>
+      </c>
       <c r="G45" s="17" t="n"/>
     </row>
     <row r="46">
@@ -1736,7 +1740,7 @@
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C46" s="8">
         <f>B46*0.124</f>
@@ -1751,7 +1755,11 @@
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="F46" s="10" t="inlineStr"/>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>Remonté de 12 à 15 € : 12 € passait sous le plancher</t>
+        </is>
+      </c>
       <c r="G46" s="11" t="n"/>
     </row>
     <row r="47" ht="22" customHeight="1">

</xml_diff>

<commit_message>
prelevements : section dediee dans la liste de vente, dates corrigees
Les quatre prelevements personnels n'apparaissaient dans la liste de
vente que sous forme d'une note en bas de la section VENDU, qui ne
citait que les Hoka et les Nike. La pompe ligne 131 et le booster
High Class n'y figuraient pas du tout.

- liste de vente : section "PRELEVE — usage personnel, HORS chiffre
  d'affaires" avec les quatre lignes, leur cout et le total de
  150,50 EUR rembourse en apport
- tableau de stock : la pompe 131 et le booster portent maintenant un
  statut "PRELEVEE 13/08" / "PRELEVE 13/08", comme les Hoka et les Nike
- registre des objets mobiliers : la date de sortie de la pompe et du
  booster etait celle de l'achat (26/07 et 03/08). Remplacee par
  13/08/2026, date de la decision, avec mention "a confirmer"

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -71,7 +71,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -96,6 +96,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F7F7F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005D6D7E"/>
       </patternFill>
     </fill>
     <fill>
@@ -150,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -186,31 +191,33 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -576,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -822,37 +829,31 @@
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>— Hoka 37⅓ et Nike Air Max Moto : PRÉLÈVEMENTS, pas des ventes</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C11" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Havaianas Slim — paire 1, N. Gulitz (Allemagne)</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="D11" s="15">
+        <f>B11*0.124</f>
+        <v/>
+      </c>
+      <c r="E11" s="16">
+        <f>B11-D11</f>
+        <v/>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Usage personnel</t>
+          <t>Vinted</t>
         </is>
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>HORS CA : ne pas déclarer les 150 €</t>
+          <t>Expédiée le 03/08 · encaissée le 10/08 · trop bas, passer à 18 €</t>
         </is>
       </c>
       <c r="H11" s="18" t="n"/>
@@ -860,7 +861,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Havaianas Slim — paire 1, N. Gulitz (Allemagne)</t>
+          <t>Havaianas Slim — paire 2, « colline_dvl »</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
@@ -884,274 +885,304 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Expédiée le 03/08 · encaissée le 10/08 · trop bas, passer à 18 €</t>
+          <t>Encaissée le 10/08 · trop bas, passer à 18 €</t>
         </is>
       </c>
       <c r="H12" s="12" t="n"/>
     </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>Havaianas Slim — paire 2, « colline_dvl »</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="n">
-        <v>14</v>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="D13" s="15">
-        <f>B13*0.124</f>
-        <v/>
-      </c>
-      <c r="E13" s="16">
-        <f>B13-D13</f>
-        <v/>
-      </c>
-      <c r="F13" s="13" t="inlineStr">
-        <is>
-          <t>Vinted</t>
-        </is>
-      </c>
-      <c r="G13" s="17" t="inlineStr">
-        <is>
-          <t>Encaissée le 10/08 · trop bas, passer à 18 €</t>
-        </is>
-      </c>
-      <c r="H13" s="18" t="n"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>🏠 PRÉLEVÉ — usage personnel, HORS chiffre d’affaires</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n"/>
+      <c r="C13" s="20" t="n"/>
+      <c r="D13" s="20" t="n"/>
+      <c r="E13" s="20" t="n"/>
+      <c r="F13" s="20" t="n"/>
+      <c r="G13" s="20" t="n"/>
+      <c r="H13" s="20" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Baskets HOKA P.37⅓ — neuves</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Gardées le 09/08</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Coût 65,37 € · aucune recette, aucune URSSAF · sortie au registre des objets mobiliers</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Baskets NIKE Air Max Moto 2K P.44,5 — neuves</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Gardées le 09/08</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>Coût 52,77 € · aucune recette, aucune URSSAF · sortie au registre des objets mobiliers</t>
+        </is>
+      </c>
+      <c r="H15" s="18" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Pompe ROBBY VP550W — ligne 131, mode auto seulement</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Gardée le 13/08</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Coût 19,41 € · la 3ᵉ pompe : deux sont à vendre, celle-ci est à toi</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Booster Pokémon High Class MEGA Dream ex M2a</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Gardé le 13/08</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>Coût 12,95 € · invendable avec profit : marché à 12,99 €</t>
+        </is>
+      </c>
+      <c r="H17" s="18" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>— TOTAL PRÉLEVÉ : 150,50 €, remboursé au compte pro en apport</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Apport, pas recette</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>NE PAS DÉCLARER À L'URSSAF · un micro-entrepreneur ne se vend pas à lui-même</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>1. URGENT — à publier cette semaine, la saison finit fin septembre</t>
         </is>
       </c>
-      <c r="B14" s="22" t="n"/>
-      <c r="C14" s="22" t="n"/>
-      <c r="D14" s="22" t="n"/>
-      <c r="E14" s="22" t="n"/>
-      <c r="F14" s="22" t="n"/>
-      <c r="G14" s="22" t="n"/>
-      <c r="H14" s="22" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="24" t="n"/>
+      <c r="F19" s="24" t="n"/>
+      <c r="G19" s="24" t="n"/>
+      <c r="H19" s="24" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Havaianas Slim fuchsia 35/36 — à l'unité, 10 restantes</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B20" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C20" s="8" t="n">
         <v>4.99</v>
       </c>
-      <c r="D15" s="9">
-        <f>B15*0.124</f>
-        <v/>
-      </c>
-      <c r="E15" s="10">
-        <f>B15-D15</f>
-        <v/>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="D20" s="9">
+        <f>B20*0.124</f>
+        <v/>
+      </c>
+      <c r="E20" s="10">
+        <f>B20-D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Vinted + Leboncoin</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>Moins cher du net 15 €/paire · 25 € par vente HORS D'ATTEINTE</t>
         </is>
       </c>
-      <c r="H15" s="12" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="H20" s="12" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>Short ba&amp;sh Fegor lightusedblue — T.34</t>
         </is>
       </c>
-      <c r="B16" s="14" t="n">
+      <c r="B21" s="14" t="n">
         <v>75</v>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C21" s="8" t="n">
         <v>11.81</v>
       </c>
-      <c r="D16" s="15">
-        <f>B16*0.124</f>
-        <v/>
-      </c>
-      <c r="E16" s="16">
-        <f>B16-D16</f>
-        <v/>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="D21" s="15">
+        <f>B21*0.124</f>
+        <v/>
+      </c>
+      <c r="E21" s="16">
+        <f>B21-D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
         <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="G16" s="17" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>Moins cher du net ~75 € Modz · plafonné, ne peut pas monter</t>
         </is>
       </c>
-      <c r="H16" s="18" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle écru</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>17.96</v>
-      </c>
-      <c r="D17" s="9">
-        <f>B17*0.124</f>
-        <v/>
-      </c>
-      <c r="E17" s="10">
-        <f>B17-D17</f>
-        <v/>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Leboncoin + Vinted</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>PRIX CORRIGÉ 19 → 34 € · neuf 37,50 € · vérifier marquage CE</t>
-        </is>
-      </c>
-      <c r="H17" s="12" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle vichy</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="n">
-        <v>34</v>
-      </c>
-      <c r="C18" s="8" t="n">
-        <v>17.96</v>
-      </c>
-      <c r="D18" s="15">
-        <f>B18*0.124</f>
-        <v/>
-      </c>
-      <c r="E18" s="16">
-        <f>B18-D18</f>
-        <v/>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>Leboncoin + Vinted</t>
-        </is>
-      </c>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>PRIX CORRIGÉ 19 → 34 € · neuf 37,50 € · vérifier marquage CE</t>
-        </is>
-      </c>
-      <c r="H18" s="18" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ écru</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="C19" s="8" t="n">
-        <v>17.96</v>
-      </c>
-      <c r="D19" s="9">
-        <f>B19*0.124</f>
-        <v/>
-      </c>
-      <c r="E19" s="10">
-        <f>B19-D19</f>
-        <v/>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>Leboncoin + Vinted</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>À publier quand le 1ᵉʳ est vendu</t>
-        </is>
-      </c>
-      <c r="H19" s="12" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ vichy</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="n">
-        <v>34</v>
-      </c>
-      <c r="C20" s="8" t="n">
-        <v>17.96</v>
-      </c>
-      <c r="D20" s="15">
-        <f>B20*0.124</f>
-        <v/>
-      </c>
-      <c r="E20" s="16">
-        <f>B20-D20</f>
-        <v/>
-      </c>
-      <c r="F20" s="13" t="inlineStr">
-        <is>
-          <t>Leboncoin + Vinted</t>
-        </is>
-      </c>
-      <c r="G20" s="17" t="inlineStr">
-        <is>
-          <t>OU les quatre en un lot à 136 € : 71,87 € en une seule vente</t>
-        </is>
-      </c>
-      <c r="H20" s="18" t="n"/>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="23" t="inlineStr">
-        <is>
-          <t>2. À PUBLIER MAINTENANT — les pièces qui rapportent</t>
-        </is>
-      </c>
-      <c r="B21" s="24" t="n"/>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="24" t="n"/>
-      <c r="F21" s="24" t="n"/>
-      <c r="G21" s="24" t="n"/>
-      <c r="H21" s="24" t="n"/>
+      <c r="H21" s="18" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Bottes Forma Legacy Waterproof — 45</t>
+          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle écru</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>159</v>
-      </c>
-      <c r="C22" s="25" t="n">
-        <v>71.53</v>
+        <v>34</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>17.96</v>
       </c>
       <c r="D22" s="9">
         <f>B22*0.124</f>
@@ -1163,12 +1194,12 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Boutique + Vinted + Leboncoin</t>
+          <t>Leboncoin + Vinted</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Neuves 172,49 € Dafy Moto</t>
+          <t>PRIX CORRIGÉ 19 → 34 € · neuf 37,50 € · vérifier marquage CE</t>
         </is>
       </c>
       <c r="H22" s="12" t="n"/>
@@ -1176,14 +1207,14 @@
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>BMW Overall ProRain unisexe noir — XL</t>
+          <t>Mrs.Ertha gilet de flottaison 3-6 ans — modèle vichy</t>
         </is>
       </c>
       <c r="B23" s="14" t="n">
-        <v>139</v>
-      </c>
-      <c r="C23" s="25" t="n">
-        <v>50.83</v>
+        <v>34</v>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>17.96</v>
       </c>
       <c r="D23" s="15">
         <f>B23*0.124</f>
@@ -1200,7 +1231,7 @@
       </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
-          <t>Neuf 170 €</t>
+          <t>PRIX CORRIGÉ 19 → 34 € · neuf 37,50 € · vérifier marquage CE</t>
         </is>
       </c>
       <c r="H23" s="18" t="n"/>
@@ -1208,14 +1239,14 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Robe Elisabetta Franchi ivoire — 46 IT / 42 FR</t>
+          <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ écru</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>99</v>
-      </c>
-      <c r="C24" s="25" t="n">
-        <v>62.42</v>
+        <v>34</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>17.96</v>
       </c>
       <c r="D24" s="9">
         <f>B24*0.124</f>
@@ -1227,12 +1258,12 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Boutique</t>
+          <t>Leboncoin + Vinted</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Défroisser avant photos</t>
+          <t>À publier quand le 1ᵉʳ est vendu</t>
         </is>
       </c>
       <c r="H24" s="12" t="n"/>
@@ -1240,14 +1271,14 @@
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>Jupe Sonia Rykiel midi twill cerises — 34</t>
+          <t>Mrs.Ertha gilet de flottaison 3-6 ans — 2ᵉ vichy</t>
         </is>
       </c>
       <c r="B25" s="14" t="n">
-        <v>99</v>
-      </c>
-      <c r="C25" s="25" t="n">
-        <v>45.07</v>
+        <v>34</v>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>17.96</v>
       </c>
       <c r="D25" s="15">
         <f>B25*0.124</f>
@@ -1259,1072 +1290,1214 @@
       </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
+          <t>Leboncoin + Vinted</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="inlineStr">
+        <is>
+          <t>OU les quatre en un lot à 136 € : 71,87 € en une seule vente</t>
+        </is>
+      </c>
+      <c r="H25" s="18" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>2. À PUBLIER MAINTENANT — les pièces qui rapportent</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="n"/>
+      <c r="C26" s="26" t="n"/>
+      <c r="D26" s="26" t="n"/>
+      <c r="E26" s="26" t="n"/>
+      <c r="F26" s="26" t="n"/>
+      <c r="G26" s="26" t="n"/>
+      <c r="H26" s="26" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Bottes Forma Legacy Waterproof — 45</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>159</v>
+      </c>
+      <c r="C27" s="27" t="n">
+        <v>71.53</v>
+      </c>
+      <c r="D27" s="9">
+        <f>B27*0.124</f>
+        <v/>
+      </c>
+      <c r="E27" s="10">
+        <f>B27-D27</f>
+        <v/>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Boutique + Vinted + Leboncoin</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>Neuves 172,49 € Dafy Moto</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>BMW Overall ProRain unisexe noir — XL</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>139</v>
+      </c>
+      <c r="C28" s="27" t="n">
+        <v>50.83</v>
+      </c>
+      <c r="D28" s="15">
+        <f>B28*0.124</f>
+        <v/>
+      </c>
+      <c r="E28" s="16">
+        <f>B28-D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>Leboncoin + Vinted</t>
+        </is>
+      </c>
+      <c r="G28" s="17" t="inlineStr">
+        <is>
+          <t>Neuf 170 €</t>
+        </is>
+      </c>
+      <c r="H28" s="18" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Robe Elisabetta Franchi ivoire — 46 IT / 42 FR</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>99</v>
+      </c>
+      <c r="C29" s="27" t="n">
+        <v>62.42</v>
+      </c>
+      <c r="D29" s="9">
+        <f>B29*0.124</f>
+        <v/>
+      </c>
+      <c r="E29" s="10">
+        <f>B29-D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="G25" s="17" t="inlineStr">
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>Défroisser avant photos</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>Jupe Sonia Rykiel midi twill cerises — 34</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>99</v>
+      </c>
+      <c r="C30" s="27" t="n">
+        <v>45.07</v>
+      </c>
+      <c r="D30" s="15">
+        <f>B30*0.124</f>
+        <v/>
+      </c>
+      <c r="E30" s="16">
+        <f>B30-D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Boutique</t>
+        </is>
+      </c>
+      <c r="G30" s="17" t="inlineStr">
         <is>
           <t>Vérifier composition sur l'étiquette</t>
         </is>
       </c>
-      <c r="H25" s="18" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="H30" s="18" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Blazer Karl Lagerfeld punto noir — 36 FR / IT 40</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n">
+      <c r="B31" s="7" t="n">
         <v>91</v>
       </c>
-      <c r="C26" s="25" t="n">
+      <c r="C31" s="27" t="n">
         <v>25.58</v>
       </c>
-      <c r="D26" s="9">
-        <f>B26*0.124</f>
-        <v/>
-      </c>
-      <c r="E26" s="10">
-        <f>B26-D26</f>
-        <v/>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="D31" s="9">
+        <f>B31*0.124</f>
+        <v/>
+      </c>
+      <c r="E31" s="10">
+        <f>B31-D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="G26" s="11" t="inlineStr">
+      <c r="G31" s="11" t="inlineStr">
         <is>
           <t>89 → 91 € · neuf dès 229 € Modalova — À RECONFIRMER avant publication</t>
         </is>
       </c>
-      <c r="H26" s="12" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="H31" s="12" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
         <is>
           <t>Adidas Predator Edge.1 TF — 48⅔ — 1ʳᵉ paire</t>
         </is>
       </c>
-      <c r="B27" s="14" t="n">
+      <c r="B32" s="14" t="n">
         <v>89</v>
       </c>
-      <c r="C27" s="25" t="n">
+      <c r="C32" s="27" t="n">
         <v>56.7</v>
       </c>
-      <c r="D27" s="15">
-        <f>B27*0.124</f>
-        <v/>
-      </c>
-      <c r="E27" s="16">
-        <f>B27-D27</f>
-        <v/>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="D32" s="15">
+        <f>B32*0.124</f>
+        <v/>
+      </c>
+      <c r="E32" s="16">
+        <f>B32-D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
         <is>
           <t>eBay + Leboncoin</t>
         </is>
       </c>
-      <c r="G27" s="17" t="inlineStr">
+      <c r="G32" s="17" t="inlineStr">
         <is>
           <t>Une annonce par paire</t>
         </is>
       </c>
-      <c r="H27" s="18" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="H32" s="18" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Adidas Predator Edge.1 TF — 48⅔ — 2ᵉ paire</t>
         </is>
       </c>
-      <c r="B28" s="7" t="n">
+      <c r="B33" s="7" t="n">
         <v>89</v>
       </c>
-      <c r="C28" s="25" t="n">
+      <c r="C33" s="27" t="n">
         <v>56.7</v>
       </c>
-      <c r="D28" s="9">
-        <f>B28*0.124</f>
-        <v/>
-      </c>
-      <c r="E28" s="10">
-        <f>B28-D28</f>
-        <v/>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="D33" s="9">
+        <f>B33*0.124</f>
+        <v/>
+      </c>
+      <c r="E33" s="10">
+        <f>B33-D33</f>
+        <v/>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>eBay + Leboncoin</t>
         </is>
       </c>
-      <c r="G28" s="11" t="inlineStr">
+      <c r="G33" s="11" t="inlineStr">
         <is>
           <t>Une annonce par paire</t>
         </is>
       </c>
-      <c r="H28" s="12" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="H33" s="12" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>Robe Sandro Noaim blanche — 40</t>
         </is>
       </c>
-      <c r="B29" s="14" t="n">
+      <c r="B34" s="14" t="n">
         <v>89</v>
       </c>
-      <c r="C29" s="25" t="n">
+      <c r="C34" s="27" t="n">
         <v>36.46</v>
       </c>
-      <c r="D29" s="15">
-        <f>B29*0.124</f>
-        <v/>
-      </c>
-      <c r="E29" s="16">
-        <f>B29-D29</f>
-        <v/>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
+      <c r="D34" s="15">
+        <f>B34*0.124</f>
+        <v/>
+      </c>
+      <c r="E34" s="16">
+        <f>B34-D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="G29" s="17" t="inlineStr">
+      <c r="G34" s="17" t="inlineStr">
         <is>
           <t>Retirer de Vinted d'abord</t>
         </is>
       </c>
-      <c r="H29" s="18" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="H34" s="18" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Plein Sport montante blanc / violet — 40</t>
         </is>
       </c>
-      <c r="B30" s="7" t="n">
+      <c r="B35" s="7" t="n">
         <v>95</v>
       </c>
-      <c r="C30" s="8" t="n">
+      <c r="C35" s="8" t="n">
         <v>23.34</v>
       </c>
-      <c r="D30" s="9">
-        <f>B30*0.124</f>
-        <v/>
-      </c>
-      <c r="E30" s="10">
-        <f>B30-D30</f>
-        <v/>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="D35" s="9">
+        <f>B35*0.124</f>
+        <v/>
+      </c>
+      <c r="E35" s="10">
+        <f>B35-D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="G30" s="11" t="inlineStr">
+      <c r="G35" s="11" t="inlineStr">
         <is>
           <t>89 → 95 € · marché ~100 € Stylight, VÉRIFIER avant de publier</t>
         </is>
       </c>
-      <c r="H30" s="12" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="H35" s="12" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
         <is>
           <t>Ballerines Hogan 186 Zeppa Fashion — 36</t>
         </is>
       </c>
-      <c r="B31" s="14" t="n">
+      <c r="B36" s="14" t="n">
         <v>79</v>
       </c>
-      <c r="C31" s="25" t="n">
+      <c r="C36" s="27" t="n">
         <v>53.05</v>
       </c>
-      <c r="D31" s="15">
-        <f>B31*0.124</f>
-        <v/>
-      </c>
-      <c r="E31" s="16">
-        <f>B31-D31</f>
-        <v/>
-      </c>
-      <c r="F31" s="13" t="inlineStr">
+      <c r="D36" s="15">
+        <f>B36*0.124</f>
+        <v/>
+      </c>
+      <c r="E36" s="16">
+        <f>B36-D36</f>
+        <v/>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="G31" s="17" t="inlineStr">
+      <c r="G36" s="17" t="inlineStr">
         <is>
           <t>Nettoyées : « aucune trace visible », PAS « neuves »</t>
         </is>
       </c>
-      <c r="H31" s="18" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="H36" s="18" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>Baskets adidas by Stella McCartney UB21 — 36</t>
         </is>
       </c>
-      <c r="B32" s="7" t="n">
+      <c r="B37" s="7" t="n">
         <v>79</v>
       </c>
-      <c r="C32" s="25" t="n">
+      <c r="C37" s="27" t="n">
         <v>27.85</v>
       </c>
-      <c r="D32" s="9">
-        <f>B32*0.124</f>
-        <v/>
-      </c>
-      <c r="E32" s="10">
-        <f>B32-D32</f>
-        <v/>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="D37" s="9">
+        <f>B37*0.124</f>
+        <v/>
+      </c>
+      <c r="E37" s="10">
+        <f>B37-D37</f>
+        <v/>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="G32" s="11" t="inlineStr">
+      <c r="G37" s="11" t="inlineStr">
         <is>
           <t>Neuf 94 € eBay.de</t>
         </is>
       </c>
-      <c r="H32" s="12" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="H37" s="12" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>Robe bustier Chiara Ferragni noire — M</t>
         </is>
       </c>
-      <c r="B33" s="14" t="n">
+      <c r="B38" s="14" t="n">
         <v>69</v>
       </c>
-      <c r="C33" s="25" t="n">
+      <c r="C38" s="27" t="n">
         <v>25.09</v>
       </c>
-      <c r="D33" s="15">
-        <f>B33*0.124</f>
-        <v/>
-      </c>
-      <c r="E33" s="16">
-        <f>B33-D33</f>
-        <v/>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
+      <c r="D38" s="15">
+        <f>B38*0.124</f>
+        <v/>
+      </c>
+      <c r="E38" s="16">
+        <f>B38-D38</f>
+        <v/>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
         <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="G33" s="17" t="inlineStr"/>
-      <c r="H33" s="18" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="G38" s="17" t="inlineStr"/>
+      <c r="H38" s="18" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>Robe Pier Antonio Gaspari bleu marine — 42</t>
         </is>
       </c>
-      <c r="B34" s="7" t="n">
+      <c r="B39" s="7" t="n">
         <v>62</v>
       </c>
-      <c r="C34" s="25" t="n">
+      <c r="C39" s="27" t="n">
         <v>25.46</v>
       </c>
-      <c r="D34" s="9">
-        <f>B34*0.124</f>
-        <v/>
-      </c>
-      <c r="E34" s="10">
-        <f>B34-D34</f>
-        <v/>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="D39" s="9">
+        <f>B39*0.124</f>
+        <v/>
+      </c>
+      <c r="E39" s="10">
+        <f>B39-D39</f>
+        <v/>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="G34" s="11" t="inlineStr">
+      <c r="G39" s="11" t="inlineStr">
         <is>
           <t>59 → 62 € · orthographe : Pier ANTONIO</t>
         </is>
       </c>
-      <c r="H34" s="12" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="H39" s="12" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>Ballerines Massimo Dutti cuir rouge — 40 IT</t>
         </is>
       </c>
-      <c r="B35" s="14" t="n">
+      <c r="B40" s="14" t="n">
         <v>61</v>
       </c>
-      <c r="C35" s="25" t="n">
+      <c r="C40" s="27" t="n">
         <v>25.87</v>
       </c>
-      <c r="D35" s="15">
-        <f>B35*0.124</f>
-        <v/>
-      </c>
-      <c r="E35" s="16">
-        <f>B35-D35</f>
-        <v/>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
+      <c r="D40" s="15">
+        <f>B40*0.124</f>
+        <v/>
+      </c>
+      <c r="E40" s="16">
+        <f>B40-D40</f>
+        <v/>
+      </c>
+      <c r="F40" s="13" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="G35" s="17" t="inlineStr">
+      <c r="G40" s="17" t="inlineStr">
         <is>
           <t>59 → 61 € · marché 70 € · pas Vinted : article neuf</t>
         </is>
       </c>
-      <c r="H35" s="18" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="H40" s="18" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>Toupies Beyblade Hasbro — LOT de 4, lot n°159</t>
         </is>
       </c>
-      <c r="B36" s="7" t="n">
+      <c r="B41" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="C36" s="25" t="n">
+      <c r="C41" s="27" t="n">
         <v>26.64</v>
       </c>
-      <c r="D36" s="9">
-        <f>B36*0.124</f>
-        <v/>
-      </c>
-      <c r="E36" s="10">
-        <f>B36-D36</f>
-        <v/>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="D41" s="9">
+        <f>B41*0.124</f>
+        <v/>
+      </c>
+      <c r="E41" s="10">
+        <f>B41-D41</f>
+        <v/>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + Vinted</t>
         </is>
       </c>
-      <c r="G36" s="11" t="inlineStr">
+      <c r="G41" s="11" t="inlineStr">
         <is>
           <t>49 → 55 € · CONFIRMER le prix des 4 toupies sur leDénicheur</t>
         </is>
       </c>
-      <c r="H36" s="12" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="H41" s="12" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>Baskets Geox gris / argent — 35</t>
         </is>
       </c>
-      <c r="B37" s="14" t="n">
+      <c r="B42" s="14" t="n">
         <v>54</v>
       </c>
-      <c r="C37" s="8" t="n">
+      <c r="C42" s="8" t="n">
         <v>23.2</v>
       </c>
-      <c r="D37" s="15">
-        <f>B37*0.124</f>
-        <v/>
-      </c>
-      <c r="E37" s="16">
-        <f>B37-D37</f>
-        <v/>
-      </c>
-      <c r="F37" s="13" t="inlineStr">
+      <c r="D42" s="15">
+        <f>B42*0.124</f>
+        <v/>
+      </c>
+      <c r="E42" s="16">
+        <f>B42-D42</f>
+        <v/>
+      </c>
+      <c r="F42" s="13" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="G37" s="17" t="inlineStr">
+      <c r="G42" s="17" t="inlineStr">
         <is>
           <t>49 → 54 € · marché 55 €, plafond atteint</t>
         </is>
       </c>
-      <c r="H37" s="18" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="H42" s="18" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>Morgan — jean bleu clair T.40</t>
         </is>
       </c>
-      <c r="B38" s="7" t="n">
+      <c r="B43" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="C38" s="8" t="n">
+      <c r="C43" s="8" t="n">
         <v>7.98</v>
       </c>
-      <c r="D38" s="9">
-        <f>B38*0.124</f>
-        <v/>
-      </c>
-      <c r="E38" s="10">
-        <f>B38-D38</f>
-        <v/>
-      </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="D43" s="9">
+        <f>B43*0.124</f>
+        <v/>
+      </c>
+      <c r="E43" s="10">
+        <f>B43-D43</f>
+        <v/>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="G38" s="11" t="inlineStr">
+      <c r="G43" s="11" t="inlineStr">
         <is>
           <t>À l'unité : 25 € par vente impossible</t>
         </is>
       </c>
-      <c r="H38" s="12" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="H43" s="12" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>Morgan — jupe marron</t>
         </is>
       </c>
-      <c r="B39" s="14" t="n">
+      <c r="B44" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="C39" s="8" t="n">
+      <c r="C44" s="8" t="n">
         <v>7.98</v>
       </c>
-      <c r="D39" s="15">
-        <f>B39*0.124</f>
-        <v/>
-      </c>
-      <c r="E39" s="16">
-        <f>B39-D39</f>
-        <v/>
-      </c>
-      <c r="F39" s="13" t="inlineStr">
+      <c r="D44" s="15">
+        <f>B44*0.124</f>
+        <v/>
+      </c>
+      <c r="E44" s="16">
+        <f>B44-D44</f>
+        <v/>
+      </c>
+      <c r="F44" s="13" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="G39" s="17" t="inlineStr"/>
-      <c r="H39" s="18" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="G44" s="17" t="inlineStr"/>
+      <c r="H44" s="18" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>Morgan — pantalon blanc T.40</t>
         </is>
       </c>
-      <c r="B40" s="7" t="n">
+      <c r="B45" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="C40" s="8" t="n">
+      <c r="C45" s="8" t="n">
         <v>4.47</v>
       </c>
-      <c r="D40" s="9">
-        <f>B40*0.124</f>
-        <v/>
-      </c>
-      <c r="E40" s="10">
-        <f>B40-D40</f>
-        <v/>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="D45" s="9">
+        <f>B45*0.124</f>
+        <v/>
+      </c>
+      <c r="E45" s="10">
+        <f>B45-D45</f>
+        <v/>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="G40" s="11" t="inlineStr"/>
-      <c r="H40" s="12" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="13" t="inlineStr">
+      <c r="G45" s="11" t="inlineStr"/>
+      <c r="H45" s="12" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
         <is>
           <t>Morgan — polo rouge à écusson doré L</t>
         </is>
       </c>
-      <c r="B41" s="14" t="n">
+      <c r="B46" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C41" s="8" t="n">
+      <c r="C46" s="8" t="n">
         <v>4.47</v>
       </c>
-      <c r="D41" s="15">
-        <f>B41*0.124</f>
-        <v/>
-      </c>
-      <c r="E41" s="16">
-        <f>B41-D41</f>
-        <v/>
-      </c>
-      <c r="F41" s="13" t="inlineStr">
+      <c r="D46" s="15">
+        <f>B46*0.124</f>
+        <v/>
+      </c>
+      <c r="E46" s="16">
+        <f>B46-D46</f>
+        <v/>
+      </c>
+      <c r="F46" s="13" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="G41" s="17" t="inlineStr"/>
-      <c r="H41" s="18" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="G46" s="17" t="inlineStr"/>
+      <c r="H46" s="18" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>Morgan — top camel lurex L</t>
         </is>
       </c>
-      <c r="B42" s="7" t="n">
+      <c r="B47" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="C42" s="8" t="n">
+      <c r="C47" s="8" t="n">
         <v>4.47</v>
       </c>
-      <c r="D42" s="9">
-        <f>B42*0.124</f>
-        <v/>
-      </c>
-      <c r="E42" s="10">
-        <f>B42-D42</f>
-        <v/>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="D47" s="9">
+        <f>B47*0.124</f>
+        <v/>
+      </c>
+      <c r="E47" s="10">
+        <f>B47-D47</f>
+        <v/>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="G42" s="11" t="inlineStr">
+      <c r="G47" s="11" t="inlineStr">
         <is>
           <t>OU les six en un lot à 98 € : 33,85 € en une seule vente</t>
         </is>
       </c>
-      <c r="H42" s="12" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="13" t="inlineStr">
+      <c r="H47" s="12" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
         <is>
           <t>Morgan — polo blanc L</t>
         </is>
       </c>
-      <c r="B43" s="14" t="n">
+      <c r="B48" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C43" s="8" t="n">
+      <c r="C48" s="8" t="n">
         <v>4.47</v>
       </c>
-      <c r="D43" s="15">
-        <f>B43*0.124</f>
-        <v/>
-      </c>
-      <c r="E43" s="16">
-        <f>B43-D43</f>
-        <v/>
-      </c>
-      <c r="F43" s="13" t="inlineStr">
+      <c r="D48" s="15">
+        <f>B48*0.124</f>
+        <v/>
+      </c>
+      <c r="E48" s="16">
+        <f>B48-D48</f>
+        <v/>
+      </c>
+      <c r="F48" s="13" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="G43" s="17" t="inlineStr"/>
-      <c r="H43" s="18" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="G48" s="17" t="inlineStr"/>
+      <c r="H48" s="18" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>Robby VP550W pompe immergée — ligne 84, occasion</t>
         </is>
       </c>
-      <c r="B44" s="7" t="n">
+      <c r="B49" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="C44" s="8" t="n">
+      <c r="C49" s="8" t="n">
         <v>3.52</v>
       </c>
-      <c r="D44" s="9">
-        <f>B44*0.124</f>
-        <v/>
-      </c>
-      <c r="E44" s="10">
-        <f>B44-D44</f>
-        <v/>
-      </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="D49" s="9">
+        <f>B49*0.124</f>
+        <v/>
+      </c>
+      <c r="E49" s="10">
+        <f>B49-D49</f>
+        <v/>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>Leboncoin, main propre</t>
         </is>
       </c>
-      <c r="G44" s="11" t="inlineStr">
+      <c r="G49" s="11" t="inlineStr">
         <is>
           <t>Neuve 54,90 € : plafonné · tester avant de publier</t>
         </is>
       </c>
-      <c r="H44" s="12" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="13" t="inlineStr">
+      <c r="H49" s="12" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="13" t="inlineStr">
         <is>
           <t>Robby VP550W pompe immergée — ligne 122, SOCLE CASSÉ</t>
         </is>
       </c>
-      <c r="B45" s="14" t="n">
+      <c r="B50" s="14" t="n">
         <v>35</v>
       </c>
-      <c r="C45" s="8" t="n">
+      <c r="C50" s="8" t="n">
         <v>2.37</v>
       </c>
-      <c r="D45" s="15">
-        <f>B45*0.124</f>
-        <v/>
-      </c>
-      <c r="E45" s="16">
-        <f>B45-D45</f>
-        <v/>
-      </c>
-      <c r="F45" s="13" t="inlineStr">
+      <c r="D50" s="15">
+        <f>B50*0.124</f>
+        <v/>
+      </c>
+      <c r="E50" s="16">
+        <f>B50-D50</f>
+        <v/>
+      </c>
+      <c r="F50" s="13" t="inlineStr">
         <is>
           <t>Leboncoin, main propre</t>
         </is>
       </c>
-      <c r="G45" s="17" t="inlineStr">
+      <c r="G50" s="17" t="inlineStr">
         <is>
           <t>DÉFAUT À DÉCLARER + photo du socle · JAMAIS d'expédition</t>
         </is>
       </c>
-      <c r="H45" s="18" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="H50" s="18" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>Toupies Beyblade Hasbro — LOT de 4, lot n°299</t>
         </is>
       </c>
-      <c r="B46" s="7" t="n">
+      <c r="B51" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="C46" s="8" t="n">
+      <c r="C51" s="8" t="n">
         <v>7.47</v>
       </c>
-      <c r="D46" s="9">
-        <f>B46*0.124</f>
-        <v/>
-      </c>
-      <c r="E46" s="10">
-        <f>B46-D46</f>
-        <v/>
-      </c>
-      <c r="F46" s="6" t="inlineStr">
+      <c r="D51" s="9">
+        <f>B51*0.124</f>
+        <v/>
+      </c>
+      <c r="E51" s="10">
+        <f>B51-D51</f>
+        <v/>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + Vinted</t>
         </is>
       </c>
-      <c r="G46" s="11" t="inlineStr">
+      <c r="G51" s="11" t="inlineStr">
         <is>
           <t>Payé 40,71 € au lieu de 21,54 € : le lot jumeau plafonne la marge</t>
         </is>
       </c>
-      <c r="H46" s="12" t="n"/>
-    </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="26" t="inlineStr">
+      <c r="H51" s="12" t="n"/>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="28" t="inlineStr">
         <is>
           <t>3. LIQUIDER — vendre pour récupérer la trésorerie, pas pour la marge</t>
         </is>
       </c>
-      <c r="B47" s="27" t="n"/>
-      <c r="C47" s="27" t="n"/>
-      <c r="D47" s="27" t="n"/>
-      <c r="E47" s="27" t="n"/>
-      <c r="F47" s="27" t="n"/>
-      <c r="G47" s="27" t="n"/>
-      <c r="H47" s="27" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="inlineStr">
+      <c r="B52" s="29" t="n"/>
+      <c r="C52" s="29" t="n"/>
+      <c r="D52" s="29" t="n"/>
+      <c r="E52" s="29" t="n"/>
+      <c r="F52" s="29" t="n"/>
+      <c r="G52" s="29" t="n"/>
+      <c r="H52" s="29" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>New Balance GS 1906 Alkaline Green — 38½</t>
         </is>
       </c>
-      <c r="B48" s="7" t="n">
+      <c r="B53" s="7" t="n">
         <v>99</v>
       </c>
-      <c r="C48" s="8" t="n">
+      <c r="C53" s="8" t="n">
         <v>8.76</v>
       </c>
-      <c r="D48" s="9">
-        <f>B48*0.124</f>
-        <v/>
-      </c>
-      <c r="E48" s="10">
-        <f>B48-D48</f>
-        <v/>
-      </c>
-      <c r="F48" s="6" t="inlineStr">
+      <c r="D53" s="9">
+        <f>B53*0.124</f>
+        <v/>
+      </c>
+      <c r="E53" s="10">
+        <f>B53-D53</f>
+        <v/>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="G48" s="11" t="inlineStr">
+      <c r="G53" s="11" t="inlineStr">
         <is>
           <t>AU-DESSUS du marché 87 € StockX — à trancher</t>
         </is>
       </c>
-      <c r="H48" s="12" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="13" t="inlineStr">
+      <c r="H53" s="12" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="13" t="inlineStr">
         <is>
           <t>Baskets Emporio Armani bleu lavande — 36</t>
         </is>
       </c>
-      <c r="B49" s="14" t="n">
+      <c r="B54" s="14" t="n">
         <v>69</v>
       </c>
-      <c r="C49" s="8" t="n">
+      <c r="C54" s="8" t="n">
         <v>6.96</v>
       </c>
-      <c r="D49" s="15">
-        <f>B49*0.124</f>
-        <v/>
-      </c>
-      <c r="E49" s="16">
-        <f>B49-D49</f>
-        <v/>
-      </c>
-      <c r="F49" s="13" t="inlineStr">
+      <c r="D54" s="15">
+        <f>B54*0.124</f>
+        <v/>
+      </c>
+      <c r="E54" s="16">
+        <f>B54-D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="13" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="G49" s="17" t="inlineStr">
+      <c r="G54" s="17" t="inlineStr">
         <is>
           <t>AU-DESSUS du marché 62 € eBay — à trancher</t>
         </is>
       </c>
-      <c r="H49" s="18" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
+      <c r="H54" s="18" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>Tommy Jeans baskets basses noir / blanc — 40</t>
         </is>
       </c>
-      <c r="B50" s="7" t="n">
+      <c r="B55" s="7" t="n">
         <v>65</v>
       </c>
-      <c r="C50" s="8" t="n">
+      <c r="C55" s="8" t="n">
         <v>2.17</v>
       </c>
-      <c r="D50" s="9">
-        <f>B50*0.124</f>
-        <v/>
-      </c>
-      <c r="E50" s="10">
-        <f>B50-D50</f>
-        <v/>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
+      <c r="D55" s="9">
+        <f>B55*0.124</f>
+        <v/>
+      </c>
+      <c r="E55" s="10">
+        <f>B55-D55</f>
+        <v/>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="G50" s="11" t="inlineStr">
+      <c r="G55" s="11" t="inlineStr">
         <is>
           <t>AU-DESSUS du marché 60 € Stylight — à trancher</t>
         </is>
       </c>
-      <c r="H50" s="12" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="13" t="inlineStr">
+      <c r="H55" s="12" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="inlineStr">
         <is>
           <t>New Balance 650 blanche montante — 44</t>
         </is>
       </c>
-      <c r="B51" s="14" t="n">
+      <c r="B56" s="14" t="n">
         <v>65</v>
       </c>
-      <c r="C51" s="8" t="n">
+      <c r="C56" s="8" t="n">
         <v>3.45</v>
       </c>
-      <c r="D51" s="15">
-        <f>B51*0.124</f>
-        <v/>
-      </c>
-      <c r="E51" s="16">
-        <f>B51-D51</f>
-        <v/>
-      </c>
-      <c r="F51" s="13" t="inlineStr">
+      <c r="D56" s="15">
+        <f>B56*0.124</f>
+        <v/>
+      </c>
+      <c r="E56" s="16">
+        <f>B56-D56</f>
+        <v/>
+      </c>
+      <c r="F56" s="13" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="G51" s="17" t="inlineStr">
+      <c r="G56" s="17" t="inlineStr">
         <is>
           <t>AU-DESSUS du marché 61 € idealo — à trancher</t>
         </is>
       </c>
-      <c r="H51" s="18" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
+      <c r="H56" s="18" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>New Balance BB80 blanc / marine — 38</t>
         </is>
       </c>
-      <c r="B52" s="7" t="n">
+      <c r="B57" s="7" t="n">
         <v>54</v>
       </c>
-      <c r="C52" s="8" t="n">
+      <c r="C57" s="8" t="n">
         <v>6.6</v>
       </c>
-      <c r="D52" s="9">
-        <f>B52*0.124</f>
-        <v/>
-      </c>
-      <c r="E52" s="10">
-        <f>B52-D52</f>
-        <v/>
-      </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="D57" s="9">
+        <f>B57*0.124</f>
+        <v/>
+      </c>
+      <c r="E57" s="10">
+        <f>B57-D57</f>
+        <v/>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="G52" s="11" t="inlineStr">
+      <c r="G57" s="11" t="inlineStr">
         <is>
           <t>Marché 54,99 € idealo : plafond atteint</t>
         </is>
       </c>
-      <c r="H52" s="12" t="n"/>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="26" t="inlineStr">
+      <c r="H57" s="12" t="n"/>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="28" t="inlineStr">
         <is>
           <t>5. POKÉMON — import du Japon, marges minces</t>
         </is>
       </c>
-      <c r="B53" s="27" t="n"/>
-      <c r="C53" s="27" t="n"/>
-      <c r="D53" s="27" t="n"/>
-      <c r="E53" s="27" t="n"/>
-      <c r="F53" s="27" t="n"/>
-      <c r="G53" s="27" t="n"/>
-      <c r="H53" s="27" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+      <c r="B58" s="29" t="n"/>
+      <c r="C58" s="29" t="n"/>
+      <c r="D58" s="29" t="n"/>
+      <c r="E58" s="29" t="n"/>
+      <c r="F58" s="29" t="n"/>
+      <c r="G58" s="29" t="n"/>
+      <c r="H58" s="29" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>Boosters Nihil Zero M3 — LOT de 15, n°1</t>
         </is>
       </c>
-      <c r="B54" s="7" t="n">
+      <c r="B59" s="7" t="n">
         <v>49</v>
       </c>
-      <c r="C54" s="8" t="n">
+      <c r="C59" s="8" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="D54" s="9">
-        <f>B54*0.124</f>
-        <v/>
-      </c>
-      <c r="E54" s="10">
-        <f>B54-D54</f>
-        <v/>
-      </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="D59" s="9">
+        <f>B59*0.124</f>
+        <v/>
+      </c>
+      <c r="E59" s="10">
+        <f>B59-D59</f>
+        <v/>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>Leboncoin, main propre</t>
         </is>
       </c>
-      <c r="G54" s="11" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr">
         <is>
           <t>PHOTOGRAPHIER LE BLISTER SCELLÉ avant d'ouvrir la box</t>
         </is>
       </c>
-      <c r="H54" s="12" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="13" t="inlineStr">
+      <c r="H59" s="12" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
         <is>
           <t>Boosters Nihil Zero M3 — LOT de 15, n°2</t>
         </is>
       </c>
-      <c r="B55" s="14" t="n">
+      <c r="B60" s="14" t="n">
         <v>49</v>
       </c>
-      <c r="C55" s="8" t="n">
+      <c r="C60" s="8" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="D55" s="15">
-        <f>B55*0.124</f>
-        <v/>
-      </c>
-      <c r="E55" s="16">
-        <f>B55-D55</f>
-        <v/>
-      </c>
-      <c r="F55" s="13" t="inlineStr">
+      <c r="D60" s="15">
+        <f>B60*0.124</f>
+        <v/>
+      </c>
+      <c r="E60" s="16">
+        <f>B60-D60</f>
+        <v/>
+      </c>
+      <c r="F60" s="13" t="inlineStr">
         <is>
           <t>Leboncoin, main propre</t>
         </is>
       </c>
-      <c r="G55" s="17" t="inlineStr">
+      <c r="G60" s="17" t="inlineStr">
         <is>
           <t>« Boosters non pesés, non triés » dans l'annonce</t>
         </is>
       </c>
-      <c r="H55" s="18" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+      <c r="H60" s="18" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t>Boosters MEGA Storm Emeralda M6 — LOT de 2</t>
         </is>
       </c>
-      <c r="B56" s="7" t="n">
+      <c r="B61" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="C56" s="8" t="n">
+      <c r="C61" s="8" t="n">
         <v>3.9</v>
       </c>
-      <c r="D56" s="9">
-        <f>B56*0.124</f>
-        <v/>
-      </c>
-      <c r="E56" s="10">
-        <f>B56-D56</f>
-        <v/>
-      </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="D61" s="9">
+        <f>B61*0.124</f>
+        <v/>
+      </c>
+      <c r="E61" s="10">
+        <f>B61-D61</f>
+        <v/>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
         <is>
           <t>Leboncoin, main propre</t>
         </is>
       </c>
-      <c r="G56" s="11" t="inlineStr">
+      <c r="G61" s="11" t="inlineStr">
         <is>
           <t>Set sorti le 31/07/2026, forte demande</t>
         </is>
       </c>
-      <c r="H56" s="12" t="n"/>
-    </row>
-    <row r="57" ht="22" customHeight="1">
-      <c r="A57" s="28" t="inlineStr">
+      <c r="H61" s="12" t="n"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="30" t="inlineStr">
         <is>
           <t>4. PLUS TARD — ne pas publier maintenant</t>
         </is>
       </c>
-      <c r="B57" s="29" t="n"/>
-      <c r="C57" s="29" t="n"/>
-      <c r="D57" s="29" t="n"/>
-      <c r="E57" s="29" t="n"/>
-      <c r="F57" s="29" t="n"/>
-      <c r="G57" s="29" t="n"/>
-      <c r="H57" s="29" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="B62" s="31" t="n"/>
+      <c r="C62" s="31" t="n"/>
+      <c r="D62" s="31" t="n"/>
+      <c r="E62" s="31" t="n"/>
+      <c r="F62" s="31" t="n"/>
+      <c r="G62" s="31" t="n"/>
+      <c r="H62" s="31" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>Lot 20 sandales et tongs — EN LOT</t>
         </is>
       </c>
-      <c r="B58" s="7" t="n">
+      <c r="B63" s="7" t="n">
         <v>199</v>
       </c>
-      <c r="C58" s="25" t="n">
+      <c r="C63" s="27" t="n">
         <v>115.25</v>
       </c>
-      <c r="D58" s="9">
-        <f>B58*0.124</f>
-        <v/>
-      </c>
-      <c r="E58" s="10">
-        <f>B58-D58</f>
-        <v/>
-      </c>
-      <c r="F58" s="6" t="inlineStr">
+      <c r="D63" s="9">
+        <f>B63*0.124</f>
+        <v/>
+      </c>
+      <c r="E63" s="10">
+        <f>B63-D63</f>
+        <v/>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
         <is>
           <t>Leboncoin B2B</t>
         </is>
       </c>
-      <c r="G58" s="11" t="inlineStr">
+      <c r="G63" s="11" t="inlineStr">
         <is>
           <t>FÉVRIER-MARS, quand le revendeur prépare l'été</t>
         </is>
       </c>
-      <c r="H58" s="12" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="13" t="inlineStr">
+      <c r="H63" s="12" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="13" t="inlineStr">
         <is>
           <t>Adidas Yeezy 700 V3 Mono Safflower — 38</t>
         </is>
       </c>
-      <c r="B59" s="14" t="n">
+      <c r="B64" s="14" t="n">
         <v>105</v>
       </c>
-      <c r="C59" s="25" t="n">
+      <c r="C64" s="27" t="n">
         <v>26.61</v>
       </c>
-      <c r="D59" s="15">
-        <f>B59*0.124</f>
-        <v/>
-      </c>
-      <c r="E59" s="16">
-        <f>B59-D59</f>
-        <v/>
-      </c>
-      <c r="F59" s="13" t="inlineStr">
+      <c r="D64" s="15">
+        <f>B64*0.124</f>
+        <v/>
+      </c>
+      <c r="E64" s="16">
+        <f>B64-D64</f>
+        <v/>
+      </c>
+      <c r="F64" s="13" t="inlineStr">
         <is>
           <t>Vinted</t>
         </is>
       </c>
-      <c r="G59" s="17" t="inlineStr">
+      <c r="G64" s="17" t="inlineStr">
         <is>
           <t>Neuve 140 € wehaveit.fr · prix valable SI l'authentification passe</t>
         </is>
       </c>
-      <c r="H59" s="18" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="30" t="inlineStr">
+      <c r="H64" s="18" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="32" t="inlineStr">
         <is>
           <t>TOTAL — 48 annonces chiffrées</t>
         </is>
       </c>
-      <c r="B60" s="31">
-        <f>B6+B7+B8+B9+B10+B12+B13+B15+B16+B17+B18+B19+B20+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36+B37+B38+B39+B40+B41+B42+B43+B44+B45+B46+B48+B49+B50+B51+B52+B54+B55+B56+B58+B59</f>
-        <v/>
-      </c>
-      <c r="C60" s="31">
-        <f>C6+C7+C8+C9+C10+C12+C13+C15+C16+C17+C18+C19+C20+C22+C23+C24+C25+C26+C27+C28+C29+C30+C31+C32+C33+C34+C35+C36+C37+C38+C39+C40+C41+C42+C43+C44+C45+C46+C48+C49+C50+C51+C52+C54+C55+C56+C58+C59</f>
-        <v/>
-      </c>
-      <c r="D60" s="32">
-        <f>B60*0.124</f>
-        <v/>
-      </c>
-      <c r="E60" s="31">
-        <f>B60-D60</f>
-        <v/>
-      </c>
-      <c r="F60" s="33" t="n"/>
-      <c r="G60" s="33" t="n"/>
-      <c r="H60" s="33" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="B65" s="33">
+        <f>B6+B7+B8+B9+B10+B11+B12+B20+B21+B22+B23+B24+B25+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36+B37+B38+B39+B40+B41+B42+B43+B44+B45+B46+B47+B48+B49+B50+B51+B53+B54+B55+B56+B57+B59+B60+B61+B63+B64</f>
+        <v/>
+      </c>
+      <c r="C65" s="33">
+        <f>C6+C7+C8+C9+C10+C11+C12+C20+C21+C22+C23+C24+C25+C27+C28+C29+C30+C31+C32+C33+C34+C35+C36+C37+C38+C39+C40+C41+C42+C43+C44+C45+C46+C47+C48+C49+C50+C51+C53+C54+C55+C56+C57+C59+C60+C61+C63+C64</f>
+        <v/>
+      </c>
+      <c r="D65" s="34">
+        <f>B65*0.124</f>
+        <v/>
+      </c>
+      <c r="E65" s="33">
+        <f>B65-D65</f>
+        <v/>
+      </c>
+      <c r="F65" s="35" t="n"/>
+      <c r="G65" s="35" t="n"/>
+      <c r="H65" s="35" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>MARGE / VENTE en vert : l'objectif de 25 € par vente est atteint. En rouge : le prix de rue plafonne, il ne peut pas l'être.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>Règle : ces prix sont calés SOUS le moins cher trouvé sur Internet. Quatre lignes en « Liquider » sont au-dessus — décision à prendre.</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>URSSAF = 12,3 % de cotisations + 0,1 % de CFP, calculé sur le prix de vente encaissé. À mettre de côté à chaque vente, pas à la fin du trimestre.</t>
         </is>

</xml_diff>

<commit_message>
correction : T-shirt Balenciaga vendu 155 EUR, pas 135 EUR
Meme cascade que la correction Armani Exchange precedente,
sur la vente a Mme Aouimeur Siham (09/08/2026, especes) :

- facture n 2026-001 : ligne T-shirt 135 -> 155 EUR, total client
  325 -> 345 EUR
- livre des recettes, registre des objets mobiliers, classeur de
  stock, liste de vente : prix et marge corriges
  (marge +2,49 -> +20,01 EUR, la plus faible marge du lot devient
  la meilleure)
- tableau de bord : CA encaisse 353 -> 373 EUR, URSSAF
  43,77 -> 46,25 EUR, marge totale 31,70 -> 49,21 EUR, total
  credite compte pro 559,82 -> 579,82 EUR, disponible
  516,05 -> 533,57 EUR, retour total 2571,12 -> 2588,64 EUR
- annonces.md : toutes les occurrences mises a jour, note de
  correction ajoutee a la suite de celle sur la veste Armani

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -655,7 +655,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>✅ VENDU — 353 € encaissés de clients réels</t>
+          <t>✅ VENDU — 373 € encaissés de clients réels</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -673,10 +673,10 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>2.49</v>
+        <v>20.01</v>
       </c>
       <c r="D6" s="9">
         <f>B6*0.124</f>
@@ -693,7 +693,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Encaissé le 09/08 · marge +2,49 € seulement</t>
+          <t>Encaissé le 09/08 · corrigé 135 → 155 €</t>
         </is>
       </c>
       <c r="H6" s="12" t="n"/>

</xml_diff>

<commit_message>
Liste de vente mise à jour : ventes, prélèvements, Pokémon, nouvel achat
Reprend tout ce qui a bougé depuis la dernière mise à jour du fichier
(15/08), resté en retard sur les autres documents :

- VENDU : total encaissé 373 € → 473 € (Salomon encaissée le 23/08, note
  mise à jour).
- PRÉLEVÉ : le booster Pokémon High Class MEGA Dream ex sort de la liste
  (jamais réintégré, reste hors activité) ; le vidéoprojecteur Philips
  NeoPix 110 y entre à sa place. Total prélevé 150,50 € → 187,95 €.
- POKÉMON : les deux lots de 15 boosters Nihil Zero fusionnés en une
  seule annonce, la box scellée entière à 89 € (au lieu de 49 € × 2) ;
  canal précisé « compte professionnel ».
- Nouvelle section « 6. INFORMATIQUE » : unité centrale gaming Acer
  G3-605, coût 88,20 €, marquée à tarifer.
- Havaianas : prix jamais reporté ici après sa révision du 16/08 —
  corrigé de 18 € à 16 € (ventes déjà faites et annonce à venir).
- Ligne TOTAL recalculée pour la nouvelle liste de cellules.
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -655,7 +655,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>✅ VENDU — 373 € encaissés de clients réels</t>
+          <t>✅ VENDU — 473 € encaissés de clients réels</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -725,7 +725,7 @@
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>Vendue le 12/08 · EXPÉDIÉE le 14/08, locker Mondial Relay · en attente d'encaissement</t>
+          <t>Vendue le 12/08 · EXPÉDIÉE le 14/08, locker Mondial Relay · ENCAISSÉE le 23/08</t>
         </is>
       </c>
       <c r="H7" s="18" t="n"/>
@@ -853,7 +853,7 @@
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>Expédiée le 03/08 · encaissée le 10/08 · trop bas, passer à 18 €</t>
+          <t>Expédiée le 03/08 · encaissée le 10/08 · trop bas, passer à 16 €</t>
         </is>
       </c>
       <c r="H11" s="18" t="n"/>
@@ -885,7 +885,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Encaissée le 10/08 · trop bas, passer à 18 €</t>
+          <t>Encaissée le 10/08 · trop bas, passer à 16 €</t>
         </is>
       </c>
       <c r="H12" s="12" t="n"/>
@@ -1021,7 +1021,7 @@
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Booster Pokémon High Class MEGA Dream ex M2a</t>
+          <t>Vidéoprojecteur PHILIPS NeoPix 110 — très bon état, testé</t>
         </is>
       </c>
       <c r="B17" s="22" t="inlineStr">
@@ -1046,12 +1046,12 @@
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Gardé le 13/08</t>
+          <t>Gardé le 23/08</t>
         </is>
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>Coût 12,95 € · invendable avec profit : marché à 12,99 €</t>
+          <t>Coût 50,40 € · facture FB2026-49549 · aucune recette, aucune URSSAF · sortie au registre des objets mobiliers</t>
         </is>
       </c>
       <c r="H17" s="18" t="n"/>
@@ -1059,7 +1059,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>— TOTAL PRÉLEVÉ : 150,50 €, remboursé au compte pro en apport</t>
+          <t>— TOTAL PRÉLEVÉ : 187,95 €, remboursé au compte pro en apport</t>
         </is>
       </c>
       <c r="B18" s="21" t="inlineStr">
@@ -1115,10 +1115,10 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>4.99</v>
+        <v>3.25</v>
       </c>
       <c r="D20" s="9">
         <f>B20*0.124</f>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Moins cher du net 15 €/paire · 25 € par vente HORS D'ATTEINTE</t>
+          <t>PRIX REVU le 16/08 (18 → 16 €) · moins cher du net 15-16 € · 25 € par vente HORS D'ATTEINTE</t>
         </is>
       </c>
       <c r="H20" s="12" t="n"/>
@@ -2285,14 +2285,14 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>Boosters Nihil Zero M3 — LOT de 15, n°1</t>
+          <t>Display Pokémon Nihil Zero M3 — box scellée entière, 30 boosters</t>
         </is>
       </c>
       <c r="B59" s="7" t="n">
-        <v>49</v>
+        <v>89</v>
       </c>
       <c r="C59" s="8" t="n">
-        <v>8.300000000000001</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="D59" s="9">
         <f>B59*0.124</f>
@@ -2304,46 +2304,24 @@
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin, main propre</t>
+          <t>Compte professionnel — Leboncoin</t>
         </is>
       </c>
       <c r="G59" s="11" t="inlineStr">
         <is>
-          <t>PHOTOGRAPHIER LE BLISTER SCELLÉ avant d'ouvrir la box</t>
+          <t>Vendue scellée, pas en lots — SCELLÉ = preuve non pesé/trié, photo du blister avant envoi</t>
         </is>
       </c>
       <c r="H59" s="12" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="13" t="inlineStr">
-        <is>
-          <t>Boosters Nihil Zero M3 — LOT de 15, n°2</t>
-        </is>
-      </c>
-      <c r="B60" s="14" t="n">
-        <v>49</v>
-      </c>
-      <c r="C60" s="8" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="D60" s="15">
-        <f>B60*0.124</f>
-        <v/>
-      </c>
-      <c r="E60" s="16">
-        <f>B60-D60</f>
-        <v/>
-      </c>
-      <c r="F60" s="13" t="inlineStr">
-        <is>
-          <t>Leboncoin, main propre</t>
-        </is>
-      </c>
-      <c r="G60" s="17" t="inlineStr">
-        <is>
-          <t>« Boosters non pesés, non triés » dans l'annonce</t>
-        </is>
-      </c>
+      <c r="A60" s="13" t="n"/>
+      <c r="B60" s="14" t="n"/>
+      <c r="C60" s="8" t="n"/>
+      <c r="D60" s="15" t="n"/>
+      <c r="E60" s="16" t="n"/>
+      <c r="F60" s="13" t="n"/>
+      <c r="G60" s="17" t="n"/>
       <c r="H60" s="18" t="n"/>
     </row>
     <row r="61">
@@ -2368,7 +2346,7 @@
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin, main propre</t>
+          <t>Compte professionnel — Leboncoin</t>
         </is>
       </c>
       <c r="G61" s="11" t="inlineStr">
@@ -2457,47 +2435,99 @@
       <c r="H64" s="18" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="32" t="inlineStr">
-        <is>
-          <t>TOTAL — 48 annonces chiffrées</t>
-        </is>
-      </c>
-      <c r="B65" s="33">
-        <f>B6+B7+B8+B9+B10+B11+B12+B20+B21+B22+B23+B24+B25+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36+B37+B38+B39+B40+B41+B42+B43+B44+B45+B46+B47+B48+B49+B50+B51+B53+B54+B55+B56+B57+B59+B60+B61+B63+B64</f>
-        <v/>
-      </c>
-      <c r="C65" s="33">
-        <f>C6+C7+C8+C9+C10+C11+C12+C20+C21+C22+C23+C24+C25+C27+C28+C29+C30+C31+C32+C33+C34+C35+C36+C37+C38+C39+C40+C41+C42+C43+C44+C45+C46+C47+C48+C49+C50+C51+C53+C54+C55+C56+C57+C59+C60+C61+C63+C64</f>
-        <v/>
-      </c>
-      <c r="D65" s="34">
-        <f>B65*0.124</f>
-        <v/>
-      </c>
-      <c r="E65" s="33">
-        <f>B65-D65</f>
-        <v/>
-      </c>
-      <c r="F65" s="35" t="n"/>
-      <c r="G65" s="35" t="n"/>
-      <c r="H65" s="35" t="n"/>
+      <c r="A65" s="30" t="inlineStr">
+        <is>
+          <t>6. INFORMATIQUE — hors périmètre mode, pas encore tarifé</t>
+        </is>
+      </c>
+      <c r="B65" s="31" t="n"/>
+      <c r="C65" s="31" t="n"/>
+      <c r="D65" s="31" t="n"/>
+      <c r="E65" s="31" t="n"/>
+      <c r="F65" s="31" t="n"/>
+      <c r="G65" s="31" t="n"/>
+      <c r="H65" s="31" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>Unité centrale gaming Acer Predator G3-605 — i7-4790, GTX 980, 16 Go RAM</t>
+        </is>
+      </c>
+      <c r="B66" s="21" t="inlineStr">
+        <is>
+          <t>à tarifer</t>
+        </is>
+      </c>
+      <c r="C66" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D66" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>Leboncoin informatique / eBay — pas la boutique</t>
+        </is>
+      </c>
+      <c r="G66" s="11" t="inlineStr">
+        <is>
+          <t>Coût 88,20 € · facture FB2026-49549 · relever le marché avant de fixer un prix</t>
+        </is>
+      </c>
+      <c r="H66" s="12" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>MARGE / VENTE en vert : l'objectif de 25 € par vente est atteint. En rouge : le prix de rue plafonne, il ne peut pas l'être.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>Règle : ces prix sont calés SOUS le moins cher trouvé sur Internet. Quatre lignes en « Liquider » sont au-dessus — décision à prendre.</t>
-        </is>
-      </c>
+      <c r="A67" s="32" t="inlineStr">
+        <is>
+          <t>TOTAL — 47 annonces chiffrées</t>
+        </is>
+      </c>
+      <c r="B67" s="33">
+        <f>B6+B7+B8+B9+B10+B11+B12+B20+B21+B22+B23+B24+B25+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36+B37+B38+B39+B40+B41+B42+B43+B44+B45+B46+B47+B48+B49+B50+B51+B53+B54+B55+B56+B57+B59+B61+B63+B64</f>
+        <v/>
+      </c>
+      <c r="C67" s="33">
+        <f>C6+C7+C8+C9+C10+C11+C12+C20+C21+C22+C23+C24+C25+C27+C28+C29+C30+C31+C32+C33+C34+C35+C36+C37+C38+C39+C40+C41+C42+C43+C44+C45+C46+C47+C48+C49+C50+C51+C53+C54+C55+C56+C57+C59+C61+C63+C64</f>
+        <v/>
+      </c>
+      <c r="D67" s="34">
+        <f>B67*0.124</f>
+        <v/>
+      </c>
+      <c r="E67" s="33">
+        <f>B67-D67</f>
+        <v/>
+      </c>
+      <c r="F67" s="35" t="n"/>
+      <c r="G67" s="35" t="n"/>
+      <c r="H67" s="35" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>MARGE / VENTE en vert : l'objectif de 25 € par vente est atteint. En rouge : le prix de rue plafonne, il ne peut pas l'être.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Règle : ces prix sont calés SOUS le moins cher trouvé sur Internet. Quatre lignes en « Liquider » sont au-dessus — décision à prendre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>URSSAF = 12,3 % de cotisations + 0,1 % de CFP, calculé sur le prix de vente encaissé. À mettre de côté à chaque vente, pas à la fin du trimestre.</t>
         </is>

</xml_diff>